<commit_message>
Add requested-amount affordability check across all loan types
- Compare requestedAmount against a simplified, deterministic
  affordability estimate derived from documented income (auto/
  personal) or documented annual revenue (small business) —
  advisory only, never an auto-decline, consistent with the
  existing human-review guarantee
- Surface warning-level flags (not just hard mismatches) at the
  application list level so an officer's queue actually reflects them
- Fix toLocaleString() rendering non-US digit grouping depending on
  server/browser locale (e.g. $3,40,000 instead of $340,000) across
  backend and frontend
- Update policy docs, FAQ, test-question bank, demo script, and the
  task tracker to match

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LoanLensAI_Development_Task_Tracker.xlsx
+++ b/docs/LoanLensAI_Development_Task_Tracker.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$F$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$F$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -668,15 +668,15 @@
     </row>
     <row r="13">
       <c r="A13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="D13" s="7">
@@ -725,15 +725,15 @@
         </is>
       </c>
       <c r="B18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A18,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A18,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A18,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A18,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A18,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A18,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E18" s="10">
@@ -748,15 +748,15 @@
         </is>
       </c>
       <c r="B19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A19,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A19,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A19,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A19,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A19,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A19,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E19" s="10">
@@ -771,15 +771,15 @@
         </is>
       </c>
       <c r="B20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A20,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A20,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A20,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A20,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A20,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A20,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E20" s="10">
@@ -794,15 +794,15 @@
         </is>
       </c>
       <c r="B21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A21,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A21,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A21,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A21,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A21,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A21,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E21" s="10">
@@ -817,15 +817,15 @@
         </is>
       </c>
       <c r="B22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A22,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A22,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A22,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A22,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A22,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A22,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E22" s="10">
@@ -840,15 +840,15 @@
         </is>
       </c>
       <c r="B23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A23,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A23,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A23,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A23,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A23,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A23,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E23" s="10">
@@ -863,15 +863,15 @@
         </is>
       </c>
       <c r="B24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A24,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A24,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A24,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A24,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A24,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A24,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E24" s="10">
@@ -886,15 +886,15 @@
         </is>
       </c>
       <c r="B25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A25,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A25,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A25,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A25,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A25,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A25,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E25" s="10">
@@ -909,15 +909,15 @@
         </is>
       </c>
       <c r="B26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A26,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A26,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A26,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A26,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A26,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A26,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E26" s="10">
@@ -932,15 +932,15 @@
         </is>
       </c>
       <c r="B27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A27,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A27,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A27,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A27,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A27,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A27,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E27" s="10">
@@ -955,15 +955,15 @@
         </is>
       </c>
       <c r="B28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A28,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A28,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A28,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A28,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A28,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A28,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E28" s="10">
@@ -978,15 +978,15 @@
         </is>
       </c>
       <c r="B29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A29,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A29,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A29,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A29,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A29,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A29,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E29" s="10">
@@ -1001,15 +1001,15 @@
         </is>
       </c>
       <c r="B30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A30,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A30,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A30,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A30,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A30,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A30,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E30" s="10">
@@ -1024,15 +1024,15 @@
         </is>
       </c>
       <c r="B31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A31,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A31,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A31,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A31,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A31,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A31,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E31" s="10">
@@ -1047,15 +1047,15 @@
         </is>
       </c>
       <c r="B32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A32,Tasks!$D$2:$D$85,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A32,Tasks!$D$2:$D$88,"Completed")</f>
         <v/>
       </c>
       <c r="C32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A32,Tasks!$D$2:$D$85,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A32,Tasks!$D$2:$D$88,"In Progress")</f>
         <v/>
       </c>
       <c r="D32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$85,$A32,Tasks!$D$2:$D$85,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$88,$A32,Tasks!$D$2:$D$88,"Not Started")</f>
         <v/>
       </c>
       <c r="E32" s="10">
@@ -1077,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1913,18 +1913,18 @@
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>One-click 'request missing document' email to borrower</t>
+          <t>Requested-amount affordability check (auto-loan, personal-loan, small-business-loan)</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E33" s="16" t="inlineStr"/>
       <c r="F33" s="17" t="inlineStr">
         <is>
-          <t>See Section 13 for the fuller self-service re-request concept from pain-point research</t>
+          <t>New — compares requestedAmount against a simplified income/revenue-based estimate; flags as Warning, never auto-declines. Not a real credit/DSCR calculation</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>6. RAG Assistant (Conversational Q&amp;A)</t>
+          <t>5. Cross-Verification Engine</t>
         </is>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>Policy corpus grounding (full corpus in context — no vector DB yet)</t>
+          <t>Warning-level flags surface at the application list level, not just inside document detail</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
@@ -1950,7 +1950,7 @@
       <c r="E34" s="16" t="inlineStr"/>
       <c r="F34" s="17" t="inlineStr">
         <is>
-          <t>services/rag.js</t>
+          <t>Fixed today — routes/documents.js previously only bumped application status to Needs Review on a hard Mismatch, so an affordability warning was invisible in the officer's list view</t>
         </is>
       </c>
     </row>
@@ -1960,12 +1960,12 @@
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>6. RAG Assistant (Conversational Q&amp;A)</t>
+          <t>5. Cross-Verification Engine</t>
         </is>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>Citation / source attribution on every answer</t>
+          <t>US currency formatting fixed regardless of server/browser locale</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
@@ -1974,7 +1974,11 @@
         </is>
       </c>
       <c r="E35" s="16" t="inlineStr"/>
-      <c r="F35" s="17" t="inlineStr"/>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>toLocaleString() was rendering $3,40,000-style grouping on non-US locales; forced to 'en-US' across backend and frontend</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="13" t="n">
@@ -1982,21 +1986,25 @@
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>6. RAG Assistant (Conversational Q&amp;A)</t>
+          <t>5. Cross-Verification Engine</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>Role-aware answers (officer vs. borrower)</t>
+          <t>One-click 'request missing document' email to borrower</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E36" s="16" t="inlineStr"/>
-      <c r="F36" s="17" t="inlineStr"/>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
+          <t>See Section 13 for the fuller self-service re-request concept from pain-point research</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="13" t="n">
@@ -2009,7 +2017,7 @@
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>Refusal behavior for out-of-corpus questions (no invented rates/policy)</t>
+          <t>Policy corpus grounding (full corpus in context — no vector DB yet)</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
@@ -2020,7 +2028,7 @@
       <c r="E37" s="16" t="inlineStr"/>
       <c r="F37" s="17" t="inlineStr">
         <is>
-          <t>Validated in data/seed/test-questions.md</t>
+          <t>services/rag.js</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2043,7 @@
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>Small-business loan Q&amp;A coverage</t>
+          <t>Citation / source attribution on every answer</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
@@ -2044,11 +2052,7 @@
         </is>
       </c>
       <c r="E38" s="16" t="inlineStr"/>
-      <c r="F38" s="17" t="inlineStr">
-        <is>
-          <t>test-questions.md items 19-23</t>
-        </is>
-      </c>
+      <c r="F38" s="17" t="inlineStr"/>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="13" t="n">
@@ -2061,20 +2065,16 @@
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>WhatsApp channel for the assistant</t>
+          <t>Role-aware answers (officer vs. borrower)</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E39" s="16" t="inlineStr"/>
-      <c r="F39" s="17" t="inlineStr">
-        <is>
-          <t>See Section 9</t>
-        </is>
-      </c>
+      <c r="F39" s="17" t="inlineStr"/>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="13" t="n">
@@ -2087,18 +2087,18 @@
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>Adverse Action notice auto-drafting (policy-grounded)</t>
+          <t>Refusal behavior for out-of-corpus questions (no invented rates/policy)</t>
         </is>
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E40" s="16" t="inlineStr"/>
       <c r="F40" s="17" t="inlineStr">
         <is>
-          <t>Recommended add-on from pain-point research — not yet scoped</t>
+          <t>Validated in data/seed/test-questions.md</t>
         </is>
       </c>
     </row>
@@ -2113,18 +2113,18 @@
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>Embeddings + vector search (scale-up path)</t>
+          <t>Small-business loan Q&amp;A coverage</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E41" s="16" t="inlineStr"/>
       <c r="F41" s="17" t="inlineStr">
         <is>
-          <t>Deliberately deferred — full corpus fits in context for the POC (ROADMAP.md)</t>
+          <t>test-questions.md items 19-23</t>
         </is>
       </c>
     </row>
@@ -2134,23 +2134,23 @@
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>7. Frontend — Screens &amp; Navigation</t>
+          <t>6. RAG Assistant (Conversational Q&amp;A)</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>Navigation shell (auth-gated stack navigation)</t>
+          <t>WhatsApp channel for the assistant</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E42" s="16" t="inlineStr"/>
       <c r="F42" s="17" t="inlineStr">
         <is>
-          <t>App.js</t>
+          <t>See Section 9</t>
         </is>
       </c>
     </row>
@@ -2160,21 +2160,25 @@
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>7. Frontend — Screens &amp; Navigation</t>
+          <t>6. RAG Assistant (Conversational Q&amp;A)</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>Login screen</t>
+          <t>Adverse Action notice auto-drafting (policy-grounded)</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E43" s="16" t="inlineStr"/>
-      <c r="F43" s="17" t="inlineStr"/>
+      <c r="F43" s="17" t="inlineStr">
+        <is>
+          <t>Recommended add-on from pain-point research — not yet scoped</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="13" t="n">
@@ -2182,23 +2186,23 @@
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>7. Frontend — Screens &amp; Navigation</t>
+          <t>6. RAG Assistant (Conversational Q&amp;A)</t>
         </is>
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>Applications list screen</t>
+          <t>Embeddings + vector search (scale-up path)</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E44" s="16" t="inlineStr"/>
       <c r="F44" s="17" t="inlineStr">
         <is>
-          <t>Officer sees all; borrower sees only their own</t>
+          <t>Deliberately deferred — full corpus fits in context for the POC (ROADMAP.md)</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2217,7 @@
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>Application detail screen (header facts + tab bar)</t>
+          <t>Navigation shell (auth-gated stack navigation)</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
@@ -2224,7 +2228,7 @@
       <c r="E45" s="16" t="inlineStr"/>
       <c r="F45" s="17" t="inlineStr">
         <is>
-          <t>Branches fact display by product type</t>
+          <t>App.js</t>
         </is>
       </c>
     </row>
@@ -2239,7 +2243,7 @@
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>Documents tab — upload + extracted fields display</t>
+          <t>Login screen</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
@@ -2261,7 +2265,7 @@
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>Verification tab — checks + missing documents</t>
+          <t>Applications list screen</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
@@ -2270,7 +2274,11 @@
         </is>
       </c>
       <c r="E47" s="16" t="inlineStr"/>
-      <c r="F47" s="17" t="inlineStr"/>
+      <c r="F47" s="17" t="inlineStr">
+        <is>
+          <t>Officer sees all; borrower sees only their own</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="13" t="n">
@@ -2283,7 +2291,7 @@
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>Assistant tab — chat UI with source chips</t>
+          <t>Application detail screen (header facts + tab bar)</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
@@ -2292,7 +2300,11 @@
         </is>
       </c>
       <c r="E48" s="16" t="inlineStr"/>
-      <c r="F48" s="17" t="inlineStr"/>
+      <c r="F48" s="17" t="inlineStr">
+        <is>
+          <t>Branches fact display by product type</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="13" t="n">
@@ -2305,7 +2317,7 @@
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>Small-business-specific detail view (business name / revenue facts)</t>
+          <t>Documents tab — upload + extracted fields display</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
@@ -2327,7 +2339,7 @@
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>Fintech-styled visual design pass</t>
+          <t>Verification tab — checks + missing documents</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
@@ -2336,11 +2348,7 @@
         </is>
       </c>
       <c r="E50" s="16" t="inlineStr"/>
-      <c r="F50" s="17" t="inlineStr">
-        <is>
-          <t>Per recent commit history</t>
-        </is>
-      </c>
+      <c r="F50" s="17" t="inlineStr"/>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="13" t="n">
@@ -2348,12 +2356,12 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>8. Synthetic Demo Data</t>
+          <t>7. Frontend — Screens &amp; Navigation</t>
         </is>
       </c>
       <c r="C51" s="15" t="inlineStr">
         <is>
-          <t>Policy corpus — 6 markdown policies</t>
+          <t>Assistant tab — chat UI with source chips</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
@@ -2362,11 +2370,7 @@
         </is>
       </c>
       <c r="E51" s="16" t="inlineStr"/>
-      <c r="F51" s="17" t="inlineStr">
-        <is>
-          <t>Application process, document checklist, income verification, auto-loan, personal-loan, FAQ</t>
-        </is>
-      </c>
+      <c r="F51" s="17" t="inlineStr"/>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="13" t="n">
@@ -2374,12 +2378,12 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>8. Synthetic Demo Data</t>
+          <t>7. Frontend — Screens &amp; Navigation</t>
         </is>
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>Small Business Loan Requirements policy</t>
+          <t>Small-business-specific detail view (business name / revenue facts)</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
@@ -2388,11 +2392,7 @@
         </is>
       </c>
       <c r="E52" s="16" t="inlineStr"/>
-      <c r="F52" s="17" t="inlineStr">
-        <is>
-          <t>data/policies/small-business-loan-requirements.md</t>
-        </is>
-      </c>
+      <c r="F52" s="17" t="inlineStr"/>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="13" t="n">
@@ -2400,12 +2400,12 @@
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>8. Synthetic Demo Data</t>
+          <t>7. Frontend — Screens &amp; Navigation</t>
         </is>
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
-          <t>Consumer demo documents — Jordan Rivera (pay stub, license, bank statement)</t>
+          <t>Fintech-styled visual design pass</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
@@ -2416,7 +2416,7 @@
       <c r="E53" s="16" t="inlineStr"/>
       <c r="F53" s="17" t="inlineStr">
         <is>
-          <t>Planted income mismatch: $4,200 vs. $5,000 stated</t>
+          <t>Per recent commit history</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>Small-business demo documents — Whitfield &amp; Co. Bakery LLC</t>
+          <t>Policy corpus — 6 markdown policies</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
@@ -2442,7 +2442,7 @@
       <c r="E54" s="16" t="inlineStr"/>
       <c r="F54" s="17" t="inlineStr">
         <is>
-          <t>Tax return, personal financial statement, business license, ownership disclosure; planted revenue mismatch ($275,400 vs. $340,000) and entity-name mismatch</t>
+          <t>Application process, document checklist, income verification, auto-loan, personal-loan, FAQ</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>Test question bank (acceptance checklist)</t>
+          <t>Small Business Loan Requirements policy</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
@@ -2468,7 +2468,7 @@
       <c r="E55" s="16" t="inlineStr"/>
       <c r="F55" s="17" t="inlineStr">
         <is>
-          <t>data/seed/test-questions.md — 23 questions across both scenarios</t>
+          <t>data/policies/small-business-loan-requirements.md</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>Demo script</t>
+          <t>Consumer demo documents — Jordan Rivera (pay stub, license, bank statement)</t>
         </is>
       </c>
       <c r="D56" s="13" t="inlineStr">
@@ -2494,7 +2494,7 @@
       <c r="E56" s="16" t="inlineStr"/>
       <c r="F56" s="17" t="inlineStr">
         <is>
-          <t>docs/DEMO_SCRIPT.md — leads with the small-business scenario</t>
+          <t>Planted income mismatch: $4,200 vs. $5,000 stated</t>
         </is>
       </c>
     </row>
@@ -2504,23 +2504,23 @@
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>9. WhatsApp Integration</t>
+          <t>8. Synthetic Demo Data</t>
         </is>
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>Meta developer app + free sandbox test number</t>
+          <t>Small-business demo documents — Whitfield &amp; Co. Bakery LLC</t>
         </is>
       </c>
       <c r="D57" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E57" s="16" t="inlineStr"/>
       <c r="F57" s="17" t="inlineStr">
         <is>
-          <t>Self-serve, free, no leadership approval needed for the demo</t>
+          <t>Tax return, personal financial statement, business license, ownership disclosure; planted revenue mismatch ($275,400 vs. $340,000) and entity-name mismatch</t>
         </is>
       </c>
     </row>
@@ -2530,21 +2530,25 @@
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>9. WhatsApp Integration</t>
+          <t>8. Synthetic Demo Data</t>
         </is>
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Webhook endpoint to receive inbound WhatsApp messages</t>
+          <t>Test question bank (acceptance checklist)</t>
         </is>
       </c>
       <c r="D58" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E58" s="16" t="inlineStr"/>
-      <c r="F58" s="17" t="inlineStr"/>
+      <c r="F58" s="17" t="inlineStr">
+        <is>
+          <t>data/seed/test-questions.md — 23 questions across both scenarios</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="13" t="n">
@@ -2552,23 +2556,23 @@
       </c>
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t>9. WhatsApp Integration</t>
+          <t>8. Synthetic Demo Data</t>
         </is>
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>Route inbound messages into the existing RAG assistant</t>
+          <t>Demo script</t>
         </is>
       </c>
       <c r="D59" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E59" s="16" t="inlineStr"/>
       <c r="F59" s="17" t="inlineStr">
         <is>
-          <t>Can reuse services/rag.js — answerQuestion()</t>
+          <t>docs/DEMO_SCRIPT.md — leads with the small-business scenario</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2587,7 @@
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>Outbound reply via WhatsApp Cloud API</t>
+          <t>Meta developer app + free sandbox test number</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
@@ -2592,7 +2596,11 @@
         </is>
       </c>
       <c r="E60" s="16" t="inlineStr"/>
-      <c r="F60" s="17" t="inlineStr"/>
+      <c r="F60" s="17" t="inlineStr">
+        <is>
+          <t>Self-serve, free, no leadership approval needed for the demo</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="13" t="n">
@@ -2605,7 +2613,7 @@
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>Production Meta Business verification</t>
+          <t>Webhook endpoint to receive inbound WhatsApp messages</t>
         </is>
       </c>
       <c r="D61" s="13" t="inlineStr">
@@ -2614,11 +2622,7 @@
         </is>
       </c>
       <c r="E61" s="16" t="inlineStr"/>
-      <c r="F61" s="17" t="inlineStr">
-        <is>
-          <t>Only needed post-demo, for a real bank pilot — not for the MVP</t>
-        </is>
-      </c>
+      <c r="F61" s="17" t="inlineStr"/>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="13" t="n">
@@ -2626,23 +2630,23 @@
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>10. Hosting &amp; Deployment</t>
+          <t>9. WhatsApp Integration</t>
         </is>
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>Render Blueprint configuration</t>
+          <t>Route inbound messages into the existing RAG assistant</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E62" s="16" t="inlineStr"/>
       <c r="F62" s="17" t="inlineStr">
         <is>
-          <t>render.yaml — backend web service + frontend static site</t>
+          <t>Can reuse services/rag.js — answerQuestion()</t>
         </is>
       </c>
     </row>
@@ -2652,25 +2656,21 @@
       </c>
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t>10. Hosting &amp; Deployment</t>
+          <t>9. WhatsApp Integration</t>
         </is>
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
-          <t>Backend deployed &amp; health-checked on Render</t>
+          <t>Outbound reply via WhatsApp Cloud API</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E63" s="16" t="inlineStr"/>
-      <c r="F63" s="17" t="inlineStr">
-        <is>
-          <t>Confirm live and reachable before demo day (/health)</t>
-        </is>
-      </c>
+      <c r="F63" s="17" t="inlineStr"/>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="13" t="n">
@@ -2678,23 +2678,23 @@
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>10. Hosting &amp; Deployment</t>
+          <t>9. WhatsApp Integration</t>
         </is>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>Frontend deployed as Render static site</t>
+          <t>Production Meta Business verification</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E64" s="16" t="inlineStr"/>
       <c r="F64" s="17" t="inlineStr">
         <is>
-          <t>Confirm Expo web export + rewrite rule are working</t>
+          <t>Only needed post-demo, for a real bank pilot — not for the MVP</t>
         </is>
       </c>
     </row>
@@ -2709,18 +2709,18 @@
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>MongoDB Atlas cluster provisioned (M0 free tier)</t>
+          <t>Render Blueprint configuration</t>
         </is>
       </c>
       <c r="D65" s="13" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E65" s="16" t="inlineStr"/>
       <c r="F65" s="17" t="inlineStr">
         <is>
-          <t>Confirm connection string + Network Access 0.0.0.0/0 are set</t>
+          <t>render.yaml — backend web service + frontend static site</t>
         </is>
       </c>
     </row>
@@ -2735,18 +2735,18 @@
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>One-shot /admin/reset endpoint for pre-demo data reset</t>
+          <t>Backend deployed &amp; health-checked on Render</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E66" s="16" t="inlineStr"/>
       <c r="F66" s="17" t="inlineStr">
         <is>
-          <t>routes/admin.js — seeds + re-indexes policies in one call</t>
+          <t>Confirm live and reachable before demo day (/health)</t>
         </is>
       </c>
     </row>
@@ -2756,23 +2756,23 @@
       </c>
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>11. Testing &amp; QA</t>
+          <t>10. Hosting &amp; Deployment</t>
         </is>
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>Manual acceptance test question bank</t>
+          <t>Frontend deployed as Render static site</t>
         </is>
       </c>
       <c r="D67" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E67" s="16" t="inlineStr"/>
       <c r="F67" s="17" t="inlineStr">
         <is>
-          <t>23 questions across consumer + small-business scenarios</t>
+          <t>Confirm Expo web export + rewrite rule are working</t>
         </is>
       </c>
     </row>
@@ -2782,21 +2782,25 @@
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>11. Testing &amp; QA</t>
+          <t>10. Hosting &amp; Deployment</t>
         </is>
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>Automated unit/integration tests</t>
+          <t>MongoDB Atlas cluster provisioned (M0 free tier)</t>
         </is>
       </c>
       <c r="D68" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E68" s="16" t="inlineStr"/>
-      <c r="F68" s="17" t="inlineStr"/>
+      <c r="F68" s="17" t="inlineStr">
+        <is>
+          <t>Confirm connection string + Network Access 0.0.0.0/0 are set</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="13" t="n">
@@ -2804,23 +2808,23 @@
       </c>
       <c r="B69" s="14" t="inlineStr">
         <is>
-          <t>11. Testing &amp; QA</t>
+          <t>10. Hosting &amp; Deployment</t>
         </is>
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>End-to-end demo rehearsal (full run-through, timed)</t>
+          <t>One-shot /admin/reset endpoint for pre-demo data reset</t>
         </is>
       </c>
       <c r="D69" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E69" s="16" t="inlineStr"/>
       <c r="F69" s="17" t="inlineStr">
         <is>
-          <t>Schedule before presentation day</t>
+          <t>routes/admin.js — seeds + re-indexes policies in one call</t>
         </is>
       </c>
     </row>
@@ -2835,16 +2839,20 @@
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Cross-browser / device check (Expo web export)</t>
+          <t>Manual acceptance test question bank</t>
         </is>
       </c>
       <c r="D70" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E70" s="16" t="inlineStr"/>
-      <c r="F70" s="17" t="inlineStr"/>
+      <c r="F70" s="17" t="inlineStr">
+        <is>
+          <t>23 questions across consumer + small-business scenarios</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="13" t="n">
@@ -2852,17 +2860,17 @@
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>12. Documentation</t>
+          <t>11. Testing &amp; QA</t>
         </is>
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>README (quick start, architecture, deploy steps)</t>
+          <t>Automated unit/integration tests</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E71" s="16" t="inlineStr"/>
@@ -2874,21 +2882,25 @@
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>12. Documentation</t>
+          <t>11. Testing &amp; QA</t>
         </is>
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>ROADMAP.md (phased build plan)</t>
+          <t>End-to-end demo rehearsal (full run-through, timed)</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E72" s="16" t="inlineStr"/>
-      <c r="F72" s="17" t="inlineStr"/>
+      <c r="F72" s="17" t="inlineStr">
+        <is>
+          <t>Schedule before presentation day</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="13" t="n">
@@ -2896,17 +2908,17 @@
       </c>
       <c r="B73" s="14" t="inlineStr">
         <is>
-          <t>12. Documentation</t>
+          <t>11. Testing &amp; QA</t>
         </is>
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>DEMO_SCRIPT.md (3-minute walkthrough)</t>
+          <t>Cross-browser / device check (Expo web export)</t>
         </is>
       </c>
       <c r="D73" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E73" s="16" t="inlineStr"/>
@@ -2923,7 +2935,7 @@
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>Development task tracker (this file)</t>
+          <t>README (quick start, architecture, deploy steps)</t>
         </is>
       </c>
       <c r="D74" s="13" t="inlineStr">
@@ -2932,11 +2944,7 @@
         </is>
       </c>
       <c r="E74" s="16" t="inlineStr"/>
-      <c r="F74" s="17" t="inlineStr">
-        <is>
-          <t>Prepared 2026-09-11, moved to Excel — update statuses as work progresses</t>
-        </is>
-      </c>
+      <c r="F74" s="17" t="inlineStr"/>
     </row>
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="13" t="n">
@@ -2944,25 +2952,21 @@
       </c>
       <c r="B75" s="14" t="inlineStr">
         <is>
-          <t>13. Real-Time Document Validation &amp; Self-Service Re-Request (DocuSense)</t>
+          <t>12. Documentation</t>
         </is>
       </c>
       <c r="C75" s="15" t="inlineStr">
         <is>
-          <t>In-browser instant document classification &amp; quality check at upload</t>
+          <t>ROADMAP.md (phased build plan)</t>
         </is>
       </c>
       <c r="D75" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr"/>
-      <c r="F75" s="17" t="inlineStr">
-        <is>
-          <t>Runs the existing extraction before submission instead of after, with immediate feedback</t>
-        </is>
-      </c>
+      <c r="F75" s="17" t="inlineStr"/>
     </row>
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="13" t="n">
@@ -2970,25 +2974,21 @@
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>13. Real-Time Document Validation &amp; Self-Service Re-Request (DocuSense)</t>
+          <t>12. Documentation</t>
         </is>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>Pre-submission completeness check (required schedules/pages present)</t>
+          <t>DEMO_SCRIPT.md (3-minute walkthrough)</t>
         </is>
       </c>
       <c r="D76" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E76" s="16" t="inlineStr"/>
-      <c r="F76" s="17" t="inlineStr">
-        <is>
-          <t>Per document type</t>
-        </is>
-      </c>
+      <c r="F76" s="17" t="inlineStr"/>
     </row>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="13" t="n">
@@ -2996,23 +2996,23 @@
       </c>
       <c r="B77" s="14" t="inlineStr">
         <is>
-          <t>13. Real-Time Document Validation &amp; Self-Service Re-Request (DocuSense)</t>
+          <t>12. Documentation</t>
         </is>
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>Blur / glare / legibility detection before accepting an upload</t>
+          <t>Development task tracker (this file)</t>
         </is>
       </c>
       <c r="D77" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E77" s="16" t="inlineStr"/>
       <c r="F77" s="17" t="inlineStr">
         <is>
-          <t>Complements existing confidence-score routing in verification.js</t>
+          <t>Prepared 2026-09-11, moved to Excel — update statuses as work progresses</t>
         </is>
       </c>
     </row>
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>Self-service secure re-upload link (SMS / magic link) on document rejection</t>
+          <t>In-browser instant document classification &amp; quality check at upload</t>
         </is>
       </c>
       <c r="D78" s="13" t="inlineStr">
@@ -3038,7 +3038,7 @@
       <c r="E78" s="16" t="inlineStr"/>
       <c r="F78" s="17" t="inlineStr">
         <is>
-          <t>Directly answers the #1 pain point from Rovo research — 'document ping-pong' / stuck Needs-Review workflows</t>
+          <t>Runs the existing extraction before submission instead of after, with immediate feedback</t>
         </is>
       </c>
     </row>
@@ -3053,7 +3053,7 @@
       </c>
       <c r="C79" s="15" t="inlineStr">
         <is>
-          <t>Auto pre-fill of underwriting review fields from extracted data</t>
+          <t>Pre-submission completeness check (required schedules/pages present)</t>
         </is>
       </c>
       <c r="D79" s="13" t="inlineStr">
@@ -3064,7 +3064,7 @@
       <c r="E79" s="16" t="inlineStr"/>
       <c r="F79" s="17" t="inlineStr">
         <is>
-          <t>Extraction already produces the data; pre-filling a review form UI is net-new</t>
+          <t>Per document type</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3074,12 @@
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>14. Multi-Party &amp; Milestone Tracking (Lending Co-Pilot)</t>
+          <t>13. Real-Time Document Validation &amp; Self-Service Re-Request (DocuSense)</t>
         </is>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>Step-by-step milestone tracker UI (Intake -&gt; Doc Verification -&gt; Underwriting -&gt; Closing -&gt; Disbursement)</t>
+          <t>Blur / glare / legibility detection before accepting an upload</t>
         </is>
       </c>
       <c r="D80" s="13" t="inlineStr">
@@ -3090,7 +3090,7 @@
       <c r="E80" s="16" t="inlineStr"/>
       <c r="F80" s="17" t="inlineStr">
         <is>
-          <t>New status model, beyond the current submitted/needs-review/approved/rejected enum</t>
+          <t>Complements existing confidence-score routing in verification.js</t>
         </is>
       </c>
     </row>
@@ -3100,12 +3100,12 @@
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>14. Multi-Party &amp; Milestone Tracking (Lending Co-Pilot)</t>
+          <t>13. Real-Time Document Validation &amp; Self-Service Re-Request (DocuSense)</t>
         </is>
       </c>
       <c r="C81" s="15" t="inlineStr">
         <is>
-          <t>Multi-party checklist — per-owner/signer verification status for business loans</t>
+          <t>Self-service secure re-upload link (SMS / magic link) on document rejection</t>
         </is>
       </c>
       <c r="D81" s="13" t="inlineStr">
@@ -3116,7 +3116,7 @@
       <c r="E81" s="16" t="inlineStr"/>
       <c r="F81" s="17" t="inlineStr">
         <is>
-          <t>Builds on the ownership-disclosure doc type; needs a per-owner sub-record, not just one applicant</t>
+          <t>Directly answers the #1 pain point from Rovo research — 'document ping-pong' / stuck Needs-Review workflows</t>
         </is>
       </c>
     </row>
@@ -3126,12 +3126,12 @@
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>14. Multi-Party &amp; Milestone Tracking (Lending Co-Pilot)</t>
+          <t>13. Real-Time Document Validation &amp; Self-Service Re-Request (DocuSense)</t>
         </is>
       </c>
       <c r="C82" s="15" t="inlineStr">
         <is>
-          <t>Shared visibility for all parties on one application</t>
+          <t>Auto pre-fill of underwriting review fields from extracted data</t>
         </is>
       </c>
       <c r="D82" s="13" t="inlineStr">
@@ -3142,7 +3142,7 @@
       <c r="E82" s="16" t="inlineStr"/>
       <c r="F82" s="17" t="inlineStr">
         <is>
-          <t>Requires multi-user access to a single application — auth model currently ties an application to one applicant email</t>
+          <t>Extraction already produces the data; pre-filling a review form UI is net-new</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3157,7 @@
       </c>
       <c r="C83" s="15" t="inlineStr">
         <is>
-          <t>Core-readiness / entity-name pre-validator earlier in the flow</t>
+          <t>Step-by-step milestone tracker UI (Intake -&gt; Doc Verification -&gt; Underwriting -&gt; Closing -&gt; Disbursement)</t>
         </is>
       </c>
       <c r="D83" s="13" t="inlineStr">
@@ -3168,7 +3168,7 @@
       <c r="E83" s="16" t="inlineStr"/>
       <c r="F83" s="17" t="inlineStr">
         <is>
-          <t>Extends the Section 5 business-name check to run at intake, before final closing</t>
+          <t>New status model, beyond the current submitted/needs-review/approved/rejected enum</t>
         </is>
       </c>
     </row>
@@ -3178,12 +3178,12 @@
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>15. Predictive Servicing (EarlyCare) — Post-MVP</t>
+          <t>14. Multi-Party &amp; Milestone Tracking (Lending Co-Pilot)</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Cash-flow dip / pre-delinquency risk detection from transaction history</t>
+          <t>Multi-party checklist — per-owner/signer verification status for business loans</t>
         </is>
       </c>
       <c r="D84" s="13" t="inlineStr">
@@ -3194,7 +3194,7 @@
       <c r="E84" s="16" t="inlineStr"/>
       <c r="F84" s="17" t="inlineStr">
         <is>
-          <t>Different lifecycle stage (servicing, not origination) — needs a transaction-history data model not in the current schema. Recommend as roadmap/vision talking point, not a 4-week build target</t>
+          <t>Builds on the ownership-disclosure doc type; needs a per-owner sub-record, not just one applicant</t>
         </is>
       </c>
     </row>
@@ -3204,12 +3204,12 @@
       </c>
       <c r="B85" s="14" t="inlineStr">
         <is>
-          <t>15. Predictive Servicing (EarlyCare) — Post-MVP</t>
+          <t>14. Multi-Party &amp; Milestone Tracking (Lending Co-Pilot)</t>
         </is>
       </c>
       <c r="C85" s="15" t="inlineStr">
         <is>
-          <t>Self-service grace period / split-payment offers</t>
+          <t>Shared visibility for all parties on one application</t>
         </is>
       </c>
       <c r="D85" s="13" t="inlineStr">
@@ -3220,13 +3220,91 @@
       <c r="E85" s="16" t="inlineStr"/>
       <c r="F85" s="17" t="inlineStr">
         <is>
+          <t>Requires multi-user access to a single application — auth model currently ties an application to one applicant email</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="30" customHeight="1">
+      <c r="A86" s="13" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="14" t="inlineStr">
+        <is>
+          <t>14. Multi-Party &amp; Milestone Tracking (Lending Co-Pilot)</t>
+        </is>
+      </c>
+      <c r="C86" s="15" t="inlineStr">
+        <is>
+          <t>Core-readiness / entity-name pre-validator earlier in the flow</t>
+        </is>
+      </c>
+      <c r="D86" s="13" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E86" s="16" t="inlineStr"/>
+      <c r="F86" s="17" t="inlineStr">
+        <is>
+          <t>Extends the Section 5 business-name check to run at intake, before final closing</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="30" customHeight="1">
+      <c r="A87" s="13" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>15. Predictive Servicing (EarlyCare) — Post-MVP</t>
+        </is>
+      </c>
+      <c r="C87" s="15" t="inlineStr">
+        <is>
+          <t>Cash-flow dip / pre-delinquency risk detection from transaction history</t>
+        </is>
+      </c>
+      <c r="D87" s="13" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E87" s="16" t="inlineStr"/>
+      <c r="F87" s="17" t="inlineStr">
+        <is>
+          <t>Different lifecycle stage (servicing, not origination) — needs a transaction-history data model not in the current schema. Recommend as roadmap/vision talking point, not a 4-week build target</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="30" customHeight="1">
+      <c r="A88" s="13" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>15. Predictive Servicing (EarlyCare) — Post-MVP</t>
+        </is>
+      </c>
+      <c r="C88" s="15" t="inlineStr">
+        <is>
+          <t>Self-service grace period / split-payment offers</t>
+        </is>
+      </c>
+      <c r="D88" s="13" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="inlineStr"/>
+      <c r="F88" s="17" t="inlineStr">
+        <is>
           <t>Same caveat as above — deprioritize for the MVP</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F85"/>
-  <conditionalFormatting sqref="D2:D85">
+  <autoFilter ref="A1:F88"/>
+  <conditionalFormatting sqref="D2:D88">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$D2="Completed"</formula>
     </cfRule>
@@ -3238,7 +3316,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Completed,In Progress,Not Started"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Turn the Apply form into a multi-step wizard; fix render.yaml service name
- NewApplicationScreen: Select Product -> Tell Us About Yourself ->
  Tell Us More About Yourself -> Disclosures & Submit, matching the
  real DAO intake step boundaries from Rovo research. Per-step
  validation blocks advancing with missing required fields instead of
  surfacing a server 400 several steps later.
- render.yaml: the deployed backend service is actually named
  "LoanLensAI" (loanlensai.onrender.com), not "loanlens-backend" as
  this file previously declared — fixed for anyone redeploying from
  scratch via Blueprint.
- Tracker updated: wizard marked Completed, 3 new test scenarios for
  step validation, age check, and consent gating.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LoanLensAI_Development_Task_Tracker.xlsx
+++ b/docs/LoanLensAI_Development_Task_Tracker.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$F$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test Scenarios'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test Scenarios'!$A$1:$G$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2697,18 +2697,18 @@
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
-          <t>Multi-step wizard for the Apply form (Select Product -&gt; Your Info -&gt; Disclosures &amp; Submit)</t>
+          <t>Multi-step wizard for the Apply form (Select Product -&gt; Tell Us About Yourself -&gt; Tell Us More About Yourself -&gt; Disclosures &amp; Submit)</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E63" s="16" t="inlineStr"/>
       <c r="F63" s="17" t="inlineStr">
         <is>
-          <t>Currently one scrollable form. Real DAO intake flows are multi-step wizards with these exact section boundaries per Rovo research — a good polish pass, not done yet</t>
+          <t>Matches the real DAO intake step boundaries from Rovo research; per-step validation blocks advancing with missing required fields, progress dots show position</t>
         </is>
       </c>
     </row>
@@ -3778,7 +3778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4492,9 +4492,114 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Apply for a loan</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Wizard step validation blocks incomplete steps</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>On 'Tell Us About Yourself' or 'Tell Us More About Yourself', leave a required field blank and tap Continue.</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>An inline error names what's missing; you stay on the same step — the wizard never lets you reach Disclosures &amp; Submit with incomplete data.</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>Prevents a 400 from the server being the first time someone learns a field was missing, several steps later — catches it at the point of entry instead.</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="inlineStr">
+        <is>
+          <t>Not yet — implemented in code, needs a live click-through once real MongoDB/Claude credentials exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>Apply for a loan</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>Under-18 date of birth is rejected</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>Enter a date of birth less than 18 years before today and submit.</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>400 error: 'Applicants must be 18 or older' — matches the eligibility text already published in every product's policy doc.</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>Closes a real gap: every policy already claimed this requirement, but nothing enforced it since there was no DOB field before this session.</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>Not yet — implemented in code, needs a live click-through once real MongoDB/Claude credentials exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="13" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Apply for a loan</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Submission is blocked without consent</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>Reach the final step without checking the disclosures/consent box.</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>Submit button is disabled (client-side); a direct API call without consentAccepted also gets a 400 server-side.</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>Matches the real 'Disclosures &amp; Submit' gate found in every DAO intake flow Rovo surfaced — belt-and-suspenders (UI + server) so it can't be bypassed by skipping the UI.</t>
+        </is>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>Not yet — implemented in code, needs a live click-through once real MongoDB/Claude credentials exist</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G20"/>
-  <conditionalFormatting sqref="G2:G20">
+  <autoFilter ref="A1:G23"/>
+  <conditionalFormatting sqref="G2:G23">
     <cfRule type="expression" priority="1" dxfId="3">
       <formula>LEFT($G2,3)="Yes"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add MOCK_AI bypass for testing without Anthropic API credits
The configured ANTHROPIC_API_KEY hit a zero credit-balance error,
blocking all document upload and assistant testing. Set MOCK_AI=true
to bypass Claude entirely:

- extraction.js: returns canned results from mockFixtures.js for the
  known seed document filenames (reproducing the exact planted
  mismatches), or a low-confidence 'unknown' for anything else —
  routes to human review same as a real illegible scan, never throws
- rag.js: returns a deterministic application-state summary instead
  of a real answer, clearly labeled as mock

Verified the Jordan Rivera pay-stub case end-to-end against the real
verification.js — mock mode reproduces the identical $5,000 vs $4,200
flag a live Claude call would produce. Off by default; must be turned
back off for the real demo, since mock answers aren't real AI output.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LoanLensAI_Development_Task_Tracker.xlsx
+++ b/docs/LoanLensAI_Development_Task_Tracker.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenarios" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$F$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test Scenarios'!$A$1:$G$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$F$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test Scenarios'!$A$1:$G$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -700,15 +700,15 @@
     </row>
     <row r="13">
       <c r="A13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="D13" s="7">
@@ -757,15 +757,15 @@
         </is>
       </c>
       <c r="B18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A18,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A18,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A18,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A18,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A18,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A18,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E18" s="10">
@@ -780,15 +780,15 @@
         </is>
       </c>
       <c r="B19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A19,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A19,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A19,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A19,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A19,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A19,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E19" s="10">
@@ -803,15 +803,15 @@
         </is>
       </c>
       <c r="B20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A20,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A20,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A20,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A20,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A20,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A20,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E20" s="10">
@@ -826,15 +826,15 @@
         </is>
       </c>
       <c r="B21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A21,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A21,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A21,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A21,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A21,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A21,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E21" s="10">
@@ -849,15 +849,15 @@
         </is>
       </c>
       <c r="B22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A22,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A22,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A22,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A22,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A22,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A22,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E22" s="10">
@@ -872,15 +872,15 @@
         </is>
       </c>
       <c r="B23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A23,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A23,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A23,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A23,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A23,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A23,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E23" s="10">
@@ -895,15 +895,15 @@
         </is>
       </c>
       <c r="B24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A24,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A24,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A24,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A24,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A24,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A24,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E24" s="10">
@@ -918,15 +918,15 @@
         </is>
       </c>
       <c r="B25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A25,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A25,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A25,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A25,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A25,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A25,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E25" s="10">
@@ -941,15 +941,15 @@
         </is>
       </c>
       <c r="B26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A26,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A26,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A26,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A26,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A26,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A26,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E26" s="10">
@@ -964,15 +964,15 @@
         </is>
       </c>
       <c r="B27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A27,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A27,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A27,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A27,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A27,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A27,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E27" s="10">
@@ -987,15 +987,15 @@
         </is>
       </c>
       <c r="B28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A28,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A28,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A28,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A28,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A28,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A28,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E28" s="10">
@@ -1010,15 +1010,15 @@
         </is>
       </c>
       <c r="B29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A29,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A29,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A29,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A29,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A29,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A29,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E29" s="10">
@@ -1033,15 +1033,15 @@
         </is>
       </c>
       <c r="B30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A30,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A30,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A30,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A30,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A30,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A30,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E30" s="10">
@@ -1056,15 +1056,15 @@
         </is>
       </c>
       <c r="B31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A31,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A31,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A31,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A31,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A31,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A31,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E31" s="10">
@@ -1079,15 +1079,15 @@
         </is>
       </c>
       <c r="B32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A32,Tasks!$D$2:$D$104,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A32,Tasks!$D$2:$D$105,"Completed")</f>
         <v/>
       </c>
       <c r="C32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A32,Tasks!$D$2:$D$104,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A32,Tasks!$D$2:$D$105,"In Progress")</f>
         <v/>
       </c>
       <c r="D32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$104,$A32,Tasks!$D$2:$D$104,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$105,$A32,Tasks!$D$2:$D$105,"Not Started")</f>
         <v/>
       </c>
       <c r="E32" s="10">
@@ -1109,7 +1109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1908,12 +1908,12 @@
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>5. Cross-Verification Engine</t>
+          <t>4. Document Intelligence (OCR / AI Extraction)</t>
         </is>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>Deterministic rule engine (not LLM — explainable/auditable)</t>
+          <t>MOCK_AI bypass — canned extraction results, no Anthropic API call</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
@@ -1924,7 +1924,7 @@
       <c r="E31" s="16" t="inlineStr"/>
       <c r="F31" s="17" t="inlineStr">
         <is>
-          <t>services/verification.js</t>
+          <t>services/mockFixtures.js + extraction.js/rag.js. Added when ANTHROPIC_API_KEY hit a zero credit-balance error blocking all testing — lets verification/live-exception/status-transition testing continue independent of API billing state. Off by default; must not be left on for the real demo</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1939,7 @@
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Name match check</t>
+          <t>Deterministic rule engine (not LLM — explainable/auditable)</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
@@ -1948,7 +1948,11 @@
         </is>
       </c>
       <c r="E32" s="16" t="inlineStr"/>
-      <c r="F32" s="17" t="inlineStr"/>
+      <c r="F32" s="17" t="inlineStr">
+        <is>
+          <t>services/verification.js</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="13" t="n">
@@ -1961,7 +1965,7 @@
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>Income match check (5% tolerance)</t>
+          <t>Name match check</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
@@ -1983,7 +1987,7 @@
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>Employer match check</t>
+          <t>Income match check (5% tolerance)</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
@@ -2005,7 +2009,7 @@
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>SSN (last 4) match check</t>
+          <t>Employer match check</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
@@ -2027,7 +2031,7 @@
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>Business name / DBA match check</t>
+          <t>SSN (last 4) match check</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
@@ -2036,11 +2040,7 @@
         </is>
       </c>
       <c r="E36" s="16" t="inlineStr"/>
-      <c r="F36" s="17" t="inlineStr">
-        <is>
-          <t>Demonstrates the entity-name-mismatch pattern found in production loan-servicing tickets</t>
-        </is>
-      </c>
+      <c r="F36" s="17" t="inlineStr"/>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="13" t="n">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>Annual business revenue match check</t>
+          <t>Business name / DBA match check</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
@@ -2062,7 +2062,11 @@
         </is>
       </c>
       <c r="E37" s="16" t="inlineStr"/>
-      <c r="F37" s="17" t="inlineStr"/>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>Demonstrates the entity-name-mismatch pattern found in production loan-servicing tickets</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="13" t="n">
@@ -2075,7 +2079,7 @@
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>Missing-document detection</t>
+          <t>Annual business revenue match check</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
@@ -2084,11 +2088,7 @@
         </is>
       </c>
       <c r="E38" s="16" t="inlineStr"/>
-      <c r="F38" s="17" t="inlineStr">
-        <is>
-          <t>missingDocuments() in verification.js</t>
-        </is>
-      </c>
+      <c r="F38" s="17" t="inlineStr"/>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="13" t="n">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>Requested-amount affordability check (auto-loan, personal-loan, small-business-loan)</t>
+          <t>Missing-document detection</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
@@ -2112,7 +2112,7 @@
       <c r="E39" s="16" t="inlineStr"/>
       <c r="F39" s="17" t="inlineStr">
         <is>
-          <t>New — compares requestedAmount against a simplified income/revenue-based estimate; flags as Warning, never auto-declines. Not a real credit/DSCR calculation</t>
+          <t>missingDocuments() in verification.js</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>Warning-level flags surface at the application list level, not just inside document detail</t>
+          <t>Requested-amount affordability check (auto-loan, personal-loan, small-business-loan)</t>
         </is>
       </c>
       <c r="D40" s="13" t="inlineStr">
@@ -2138,7 +2138,7 @@
       <c r="E40" s="16" t="inlineStr"/>
       <c r="F40" s="17" t="inlineStr">
         <is>
-          <t>Fixed today — routes/documents.js previously only bumped application status to Needs Review on a hard Mismatch, so an affordability warning was invisible in the officer's list view</t>
+          <t>New — compares requestedAmount against a simplified income/revenue-based estimate; flags as Warning, never auto-declines. Not a real credit/DSCR calculation</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>US currency formatting fixed regardless of server/browser locale</t>
+          <t>Warning-level flags surface at the application list level, not just inside document detail</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
@@ -2164,7 +2164,7 @@
       <c r="E41" s="16" t="inlineStr"/>
       <c r="F41" s="17" t="inlineStr">
         <is>
-          <t>toLocaleString() was rendering $3,40,000-style grouping on non-US locales; forced to 'en-US' across backend and frontend</t>
+          <t>Fixed today — routes/documents.js previously only bumped application status to Needs Review on a hard Mismatch, so an affordability warning was invisible in the officer's list view</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2179,7 @@
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>One-click 'request missing document' email to borrower</t>
+          <t>US currency formatting fixed regardless of server/browser locale</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
@@ -2190,7 +2190,7 @@
       <c r="E42" s="16" t="inlineStr"/>
       <c r="F42" s="17" t="inlineStr">
         <is>
-          <t>Superseded by the richer in-app live-exception + targeted self-service re-upload flow — see Section 13. No email/SMS needed; the borrower sees and fixes it directly in the app</t>
+          <t>toLocaleString() was rendering $3,40,000-style grouping on non-US locales; forced to 'en-US' across backend and frontend</t>
         </is>
       </c>
     </row>
@@ -2200,12 +2200,12 @@
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>6. RAG Assistant (Conversational Q&amp;A)</t>
+          <t>5. Cross-Verification Engine</t>
         </is>
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>Policy corpus grounding (full corpus in context — no vector DB yet)</t>
+          <t>One-click 'request missing document' email to borrower</t>
         </is>
       </c>
       <c r="D43" s="13" t="inlineStr">
@@ -2216,7 +2216,7 @@
       <c r="E43" s="16" t="inlineStr"/>
       <c r="F43" s="17" t="inlineStr">
         <is>
-          <t>services/rag.js</t>
+          <t>Superseded by the richer in-app live-exception + targeted self-service re-upload flow — see Section 13. No email/SMS needed; the borrower sees and fixes it directly in the app</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>Citation / source attribution on every answer</t>
+          <t>Policy corpus grounding (full corpus in context — no vector DB yet)</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
@@ -2240,7 +2240,11 @@
         </is>
       </c>
       <c r="E44" s="16" t="inlineStr"/>
-      <c r="F44" s="17" t="inlineStr"/>
+      <c r="F44" s="17" t="inlineStr">
+        <is>
+          <t>services/rag.js</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="13" t="n">
@@ -2253,7 +2257,7 @@
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>Role-aware answers (officer vs. borrower)</t>
+          <t>Citation / source attribution on every answer</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
@@ -2275,7 +2279,7 @@
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>Refusal behavior for out-of-corpus questions (no invented rates/policy)</t>
+          <t>Role-aware answers (officer vs. borrower)</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
@@ -2284,11 +2288,7 @@
         </is>
       </c>
       <c r="E46" s="16" t="inlineStr"/>
-      <c r="F46" s="17" t="inlineStr">
-        <is>
-          <t>Validated in data/seed/test-questions.md</t>
-        </is>
-      </c>
+      <c r="F46" s="17" t="inlineStr"/>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="13" t="n">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>Small-business loan Q&amp;A coverage</t>
+          <t>Refusal behavior for out-of-corpus questions (no invented rates/policy)</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
@@ -2312,7 +2312,7 @@
       <c r="E47" s="16" t="inlineStr"/>
       <c r="F47" s="17" t="inlineStr">
         <is>
-          <t>test-questions.md items 19-23</t>
+          <t>Validated in data/seed/test-questions.md</t>
         </is>
       </c>
     </row>
@@ -2327,18 +2327,18 @@
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>WhatsApp channel for the assistant</t>
+          <t>Small-business loan Q&amp;A coverage</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E48" s="16" t="inlineStr"/>
       <c r="F48" s="17" t="inlineStr">
         <is>
-          <t>See Section 9</t>
+          <t>test-questions.md items 19-23</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>Adverse Action notice auto-drafting (policy-grounded)</t>
+          <t>WhatsApp channel for the assistant</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
@@ -2364,7 +2364,7 @@
       <c r="E49" s="16" t="inlineStr"/>
       <c r="F49" s="17" t="inlineStr">
         <is>
-          <t>Recommended add-on from pain-point research — not yet scoped</t>
+          <t>See Section 9</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>Embeddings + vector search (scale-up path)</t>
+          <t>Adverse Action notice auto-drafting (policy-grounded)</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
@@ -2390,7 +2390,7 @@
       <c r="E50" s="16" t="inlineStr"/>
       <c r="F50" s="17" t="inlineStr">
         <is>
-          <t>Deliberately deferred — full corpus fits in context for the POC (ROADMAP.md)</t>
+          <t>Recommended add-on from pain-point research — not yet scoped</t>
         </is>
       </c>
     </row>
@@ -2400,23 +2400,23 @@
       </c>
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>7. Frontend — Screens &amp; Navigation</t>
+          <t>6. RAG Assistant (Conversational Q&amp;A)</t>
         </is>
       </c>
       <c r="C51" s="15" t="inlineStr">
         <is>
-          <t>Navigation shell (auth-gated stack navigation)</t>
+          <t>Embeddings + vector search (scale-up path)</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E51" s="16" t="inlineStr"/>
       <c r="F51" s="17" t="inlineStr">
         <is>
-          <t>App.js</t>
+          <t>Deliberately deferred — full corpus fits in context for the POC (ROADMAP.md)</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>Login screen</t>
+          <t>Navigation shell (auth-gated stack navigation)</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
@@ -2440,7 +2440,11 @@
         </is>
       </c>
       <c r="E52" s="16" t="inlineStr"/>
-      <c r="F52" s="17" t="inlineStr"/>
+      <c r="F52" s="17" t="inlineStr">
+        <is>
+          <t>App.js</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="13" t="n">
@@ -2453,7 +2457,7 @@
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
-          <t>Applications list screen</t>
+          <t>Login screen</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
@@ -2462,11 +2466,7 @@
         </is>
       </c>
       <c r="E53" s="16" t="inlineStr"/>
-      <c r="F53" s="17" t="inlineStr">
-        <is>
-          <t>Officer sees all; borrower sees only their own</t>
-        </is>
-      </c>
+      <c r="F53" s="17" t="inlineStr"/>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="13" t="n">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>Application detail screen (header facts + tab bar)</t>
+          <t>Applications list screen</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
@@ -2490,7 +2490,7 @@
       <c r="E54" s="16" t="inlineStr"/>
       <c r="F54" s="17" t="inlineStr">
         <is>
-          <t>Branches fact display by product type</t>
+          <t>Officer sees all; borrower sees only their own</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>Documents tab — upload + extracted fields display</t>
+          <t>Application detail screen (header facts + tab bar)</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
@@ -2514,7 +2514,11 @@
         </is>
       </c>
       <c r="E55" s="16" t="inlineStr"/>
-      <c r="F55" s="17" t="inlineStr"/>
+      <c r="F55" s="17" t="inlineStr">
+        <is>
+          <t>Branches fact display by product type</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="13" t="n">
@@ -2527,7 +2531,7 @@
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>Verification tab — checks + missing documents</t>
+          <t>Documents tab — upload + extracted fields display</t>
         </is>
       </c>
       <c r="D56" s="13" t="inlineStr">
@@ -2549,7 +2553,7 @@
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>Assistant tab — chat UI with source chips</t>
+          <t>Verification tab — checks + missing documents</t>
         </is>
       </c>
       <c r="D57" s="13" t="inlineStr">
@@ -2571,7 +2575,7 @@
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Small-business-specific detail view (business name / revenue facts)</t>
+          <t>Assistant tab — chat UI with source chips</t>
         </is>
       </c>
       <c r="D58" s="13" t="inlineStr">
@@ -2593,7 +2597,7 @@
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>Fintech-styled visual design pass</t>
+          <t>Small-business-specific detail view (business name / revenue facts)</t>
         </is>
       </c>
       <c r="D59" s="13" t="inlineStr">
@@ -2602,11 +2606,7 @@
         </is>
       </c>
       <c r="E59" s="16" t="inlineStr"/>
-      <c r="F59" s="17" t="inlineStr">
-        <is>
-          <t>Per recent commit history</t>
-        </is>
-      </c>
+      <c r="F59" s="17" t="inlineStr"/>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="13" t="n">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>Sign-up screen (self-registration, role picker)</t>
+          <t>Fintech-styled visual design pass</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
@@ -2630,7 +2630,7 @@
       <c r="E60" s="16" t="inlineStr"/>
       <c r="F60" s="17" t="inlineStr">
         <is>
-          <t>SignUpScreen.js</t>
+          <t>Per recent commit history</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>New Application screen ('Apply for a Loan')</t>
+          <t>Sign-up screen (self-registration, role picker)</t>
         </is>
       </c>
       <c r="D61" s="13" t="inlineStr">
@@ -2656,7 +2656,7 @@
       <c r="E61" s="16" t="inlineStr"/>
       <c r="F61" s="17" t="inlineStr">
         <is>
-          <t>NewApplicationScreen.js — product-type picker with conditional fields (consumer income/employer vs. business name/revenue), submits to POST /applications then lands on that application's Documents tab</t>
+          <t>SignUpScreen.js</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2671,7 @@
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>'New application' entry point on the borrower's Applications list</t>
+          <t>New Application screen ('Apply for a Loan')</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
@@ -2682,7 +2682,7 @@
       <c r="E62" s="16" t="inlineStr"/>
       <c r="F62" s="17" t="inlineStr">
         <is>
-          <t>Officer role doesn't see this button — they don't file applications for themselves</t>
+          <t>NewApplicationScreen.js — product-type picker with conditional fields (consumer income/employer vs. business name/revenue), submits to POST /applications then lands on that application's Documents tab</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
-          <t>Multi-step wizard for the Apply form (Select Product -&gt; Tell Us About Yourself -&gt; Tell Us More About Yourself -&gt; Disclosures &amp; Submit)</t>
+          <t>'New application' entry point on the borrower's Applications list</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
@@ -2708,7 +2708,7 @@
       <c r="E63" s="16" t="inlineStr"/>
       <c r="F63" s="17" t="inlineStr">
         <is>
-          <t>Matches the real DAO intake step boundaries from Rovo research; per-step validation blocks advancing with missing required fields, progress dots show position</t>
+          <t>Officer role doesn't see this button — they don't file applications for themselves</t>
         </is>
       </c>
     </row>
@@ -2718,12 +2718,12 @@
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>8. Synthetic Demo Data</t>
+          <t>7. Frontend — Screens &amp; Navigation</t>
         </is>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>Policy corpus — 6 markdown policies</t>
+          <t>Multi-step wizard for the Apply form (Select Product -&gt; Tell Us About Yourself -&gt; Tell Us More About Yourself -&gt; Disclosures &amp; Submit)</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
@@ -2734,7 +2734,7 @@
       <c r="E64" s="16" t="inlineStr"/>
       <c r="F64" s="17" t="inlineStr">
         <is>
-          <t>Application process, document checklist, income verification, auto-loan, personal-loan, FAQ</t>
+          <t>Matches the real DAO intake step boundaries from Rovo research; per-step validation blocks advancing with missing required fields, progress dots show position</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2749,7 @@
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>Small Business Loan Requirements policy</t>
+          <t>Policy corpus — 6 markdown policies</t>
         </is>
       </c>
       <c r="D65" s="13" t="inlineStr">
@@ -2760,7 +2760,7 @@
       <c r="E65" s="16" t="inlineStr"/>
       <c r="F65" s="17" t="inlineStr">
         <is>
-          <t>data/policies/small-business-loan-requirements.md</t>
+          <t>Application process, document checklist, income verification, auto-loan, personal-loan, FAQ</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>Consumer demo documents — Jordan Rivera (pay stub, license, bank statement)</t>
+          <t>Small Business Loan Requirements policy</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
@@ -2786,7 +2786,7 @@
       <c r="E66" s="16" t="inlineStr"/>
       <c r="F66" s="17" t="inlineStr">
         <is>
-          <t>Planted income mismatch: $4,200 vs. $5,000 stated</t>
+          <t>data/policies/small-business-loan-requirements.md</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>Small-business demo documents — Whitfield &amp; Co. Bakery LLC</t>
+          <t>Consumer demo documents — Jordan Rivera (pay stub, license, bank statement)</t>
         </is>
       </c>
       <c r="D67" s="13" t="inlineStr">
@@ -2812,7 +2812,7 @@
       <c r="E67" s="16" t="inlineStr"/>
       <c r="F67" s="17" t="inlineStr">
         <is>
-          <t>Tax return, personal financial statement, business license, ownership disclosure; planted revenue mismatch ($275,400 vs. $340,000) and entity-name mismatch</t>
+          <t>Planted income mismatch: $4,200 vs. $5,000 stated</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2827,7 @@
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>Test question bank (acceptance checklist)</t>
+          <t>Small-business demo documents — Whitfield &amp; Co. Bakery LLC</t>
         </is>
       </c>
       <c r="D68" s="13" t="inlineStr">
@@ -2838,7 +2838,7 @@
       <c r="E68" s="16" t="inlineStr"/>
       <c r="F68" s="17" t="inlineStr">
         <is>
-          <t>data/seed/test-questions.md — 23 questions across both scenarios</t>
+          <t>Tax return, personal financial statement, business license, ownership disclosure; planted revenue mismatch ($275,400 vs. $340,000) and entity-name mismatch</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>Demo script</t>
+          <t>Test question bank (acceptance checklist)</t>
         </is>
       </c>
       <c r="D69" s="13" t="inlineStr">
@@ -2864,7 +2864,7 @@
       <c r="E69" s="16" t="inlineStr"/>
       <c r="F69" s="17" t="inlineStr">
         <is>
-          <t>docs/DEMO_SCRIPT.md — leads with the small-business scenario</t>
+          <t>data/seed/test-questions.md — 23 questions across both scenarios</t>
         </is>
       </c>
     </row>
@@ -2874,23 +2874,23 @@
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>9. WhatsApp Integration</t>
+          <t>8. Synthetic Demo Data</t>
         </is>
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Meta developer app + free sandbox test number</t>
+          <t>Demo script</t>
         </is>
       </c>
       <c r="D70" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E70" s="16" t="inlineStr"/>
       <c r="F70" s="17" t="inlineStr">
         <is>
-          <t>Self-serve, free, no leadership approval needed for the demo</t>
+          <t>docs/DEMO_SCRIPT.md — leads with the small-business scenario</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>Webhook endpoint to receive inbound WhatsApp messages</t>
+          <t>Meta developer app + free sandbox test number</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
@@ -2914,7 +2914,11 @@
         </is>
       </c>
       <c r="E71" s="16" t="inlineStr"/>
-      <c r="F71" s="17" t="inlineStr"/>
+      <c r="F71" s="17" t="inlineStr">
+        <is>
+          <t>Self-serve, free, no leadership approval needed for the demo</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="13" t="n">
@@ -2927,7 +2931,7 @@
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>Route inbound messages into the existing RAG assistant</t>
+          <t>Webhook endpoint to receive inbound WhatsApp messages</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr">
@@ -2936,11 +2940,7 @@
         </is>
       </c>
       <c r="E72" s="16" t="inlineStr"/>
-      <c r="F72" s="17" t="inlineStr">
-        <is>
-          <t>Can reuse services/rag.js — answerQuestion()</t>
-        </is>
-      </c>
+      <c r="F72" s="17" t="inlineStr"/>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="13" t="n">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>Outbound reply via WhatsApp Cloud API</t>
+          <t>Route inbound messages into the existing RAG assistant</t>
         </is>
       </c>
       <c r="D73" s="13" t="inlineStr">
@@ -2962,7 +2962,11 @@
         </is>
       </c>
       <c r="E73" s="16" t="inlineStr"/>
-      <c r="F73" s="17" t="inlineStr"/>
+      <c r="F73" s="17" t="inlineStr">
+        <is>
+          <t>Can reuse services/rag.js — answerQuestion()</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="13" t="n">
@@ -2975,7 +2979,7 @@
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>Production Meta Business verification</t>
+          <t>Outbound reply via WhatsApp Cloud API</t>
         </is>
       </c>
       <c r="D74" s="13" t="inlineStr">
@@ -2984,11 +2988,7 @@
         </is>
       </c>
       <c r="E74" s="16" t="inlineStr"/>
-      <c r="F74" s="17" t="inlineStr">
-        <is>
-          <t>Only needed post-demo, for a real bank pilot — not for the MVP</t>
-        </is>
-      </c>
+      <c r="F74" s="17" t="inlineStr"/>
     </row>
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="13" t="n">
@@ -2996,23 +2996,23 @@
       </c>
       <c r="B75" s="14" t="inlineStr">
         <is>
-          <t>10. Hosting &amp; Deployment</t>
+          <t>9. WhatsApp Integration</t>
         </is>
       </c>
       <c r="C75" s="15" t="inlineStr">
         <is>
-          <t>Render Blueprint configuration</t>
+          <t>Production Meta Business verification</t>
         </is>
       </c>
       <c r="D75" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr"/>
       <c r="F75" s="17" t="inlineStr">
         <is>
-          <t>render.yaml — backend web service + frontend static site</t>
+          <t>Only needed post-demo, for a real bank pilot — not for the MVP</t>
         </is>
       </c>
     </row>
@@ -3027,18 +3027,18 @@
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>Backend deployed &amp; health-checked on Render</t>
+          <t>Render Blueprint configuration</t>
         </is>
       </c>
       <c r="D76" s="13" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E76" s="16" t="inlineStr"/>
       <c r="F76" s="17" t="inlineStr">
         <is>
-          <t>Confirm live and reachable before demo day (/health)</t>
+          <t>render.yaml — backend web service + frontend static site</t>
         </is>
       </c>
     </row>
@@ -3053,7 +3053,7 @@
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>Frontend deployed as Render static site</t>
+          <t>Backend deployed &amp; health-checked on Render</t>
         </is>
       </c>
       <c r="D77" s="13" t="inlineStr">
@@ -3064,7 +3064,7 @@
       <c r="E77" s="16" t="inlineStr"/>
       <c r="F77" s="17" t="inlineStr">
         <is>
-          <t>Confirm Expo web export + rewrite rule are working</t>
+          <t>Confirm live and reachable before demo day (/health)</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>MongoDB Atlas cluster provisioned (M0 free tier)</t>
+          <t>Frontend deployed as Render static site</t>
         </is>
       </c>
       <c r="D78" s="13" t="inlineStr">
@@ -3090,7 +3090,7 @@
       <c r="E78" s="16" t="inlineStr"/>
       <c r="F78" s="17" t="inlineStr">
         <is>
-          <t>Confirm connection string + Network Access 0.0.0.0/0 are set</t>
+          <t>Confirm Expo web export + rewrite rule are working</t>
         </is>
       </c>
     </row>
@@ -3105,18 +3105,18 @@
       </c>
       <c r="C79" s="15" t="inlineStr">
         <is>
-          <t>One-shot /admin/reset endpoint for pre-demo data reset</t>
+          <t>MongoDB Atlas cluster provisioned (M0 free tier)</t>
         </is>
       </c>
       <c r="D79" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E79" s="16" t="inlineStr"/>
       <c r="F79" s="17" t="inlineStr">
         <is>
-          <t>routes/admin.js — seeds + re-indexes policies in one call</t>
+          <t>Confirm connection string + Network Access 0.0.0.0/0 are set</t>
         </is>
       </c>
     </row>
@@ -3126,12 +3126,12 @@
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>11. Testing &amp; QA</t>
+          <t>10. Hosting &amp; Deployment</t>
         </is>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>Manual acceptance test question bank</t>
+          <t>One-shot /admin/reset endpoint for pre-demo data reset</t>
         </is>
       </c>
       <c r="D80" s="13" t="inlineStr">
@@ -3142,7 +3142,7 @@
       <c r="E80" s="16" t="inlineStr"/>
       <c r="F80" s="17" t="inlineStr">
         <is>
-          <t>23 questions across consumer + small-business scenarios</t>
+          <t>routes/admin.js — seeds + re-indexes policies in one call</t>
         </is>
       </c>
     </row>
@@ -3157,16 +3157,20 @@
       </c>
       <c r="C81" s="15" t="inlineStr">
         <is>
-          <t>Automated unit/integration tests</t>
+          <t>Manual acceptance test question bank</t>
         </is>
       </c>
       <c r="D81" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E81" s="16" t="inlineStr"/>
-      <c r="F81" s="17" t="inlineStr"/>
+      <c r="F81" s="17" t="inlineStr">
+        <is>
+          <t>23 questions across consumer + small-business scenarios</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="13" t="n">
@@ -3179,7 +3183,7 @@
       </c>
       <c r="C82" s="15" t="inlineStr">
         <is>
-          <t>End-to-end demo rehearsal (full run-through, timed)</t>
+          <t>Automated unit/integration tests</t>
         </is>
       </c>
       <c r="D82" s="13" t="inlineStr">
@@ -3188,11 +3192,7 @@
         </is>
       </c>
       <c r="E82" s="16" t="inlineStr"/>
-      <c r="F82" s="17" t="inlineStr">
-        <is>
-          <t>Schedule before presentation day</t>
-        </is>
-      </c>
+      <c r="F82" s="17" t="inlineStr"/>
     </row>
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="13" t="n">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="C83" s="15" t="inlineStr">
         <is>
-          <t>Cross-browser / device check (Expo web export)</t>
+          <t>End-to-end demo rehearsal (full run-through, timed)</t>
         </is>
       </c>
       <c r="D83" s="13" t="inlineStr">
@@ -3214,7 +3214,11 @@
         </is>
       </c>
       <c r="E83" s="16" t="inlineStr"/>
-      <c r="F83" s="17" t="inlineStr"/>
+      <c r="F83" s="17" t="inlineStr">
+        <is>
+          <t>Schedule before presentation day</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="13" t="n">
@@ -3222,17 +3226,17 @@
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>12. Documentation</t>
+          <t>11. Testing &amp; QA</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>README (quick start, architecture, deploy steps)</t>
+          <t>Cross-browser / device check (Expo web export)</t>
         </is>
       </c>
       <c r="D84" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E84" s="16" t="inlineStr"/>
@@ -3249,7 +3253,7 @@
       </c>
       <c r="C85" s="15" t="inlineStr">
         <is>
-          <t>ROADMAP.md (phased build plan)</t>
+          <t>README (quick start, architecture, deploy steps)</t>
         </is>
       </c>
       <c r="D85" s="13" t="inlineStr">
@@ -3271,7 +3275,7 @@
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>DEMO_SCRIPT.md (3-minute walkthrough)</t>
+          <t>ROADMAP.md (phased build plan)</t>
         </is>
       </c>
       <c r="D86" s="13" t="inlineStr">
@@ -3293,7 +3297,7 @@
       </c>
       <c r="C87" s="15" t="inlineStr">
         <is>
-          <t>Development task tracker (this file)</t>
+          <t>DEMO_SCRIPT.md (3-minute walkthrough)</t>
         </is>
       </c>
       <c r="D87" s="13" t="inlineStr">
@@ -3302,11 +3306,7 @@
         </is>
       </c>
       <c r="E87" s="16" t="inlineStr"/>
-      <c r="F87" s="17" t="inlineStr">
-        <is>
-          <t>Prepared 2026-09-11, moved to Excel — update statuses as work progresses</t>
-        </is>
-      </c>
+      <c r="F87" s="17" t="inlineStr"/>
     </row>
     <row r="88" ht="30" customHeight="1">
       <c r="A88" s="13" t="n">
@@ -3314,12 +3314,12 @@
       </c>
       <c r="B88" s="14" t="inlineStr">
         <is>
-          <t>13. Real-Time Document Validation &amp; Self-Service Re-Request (DocuSense)</t>
+          <t>12. Documentation</t>
         </is>
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Unified 'Action needed' list — every open issue (missing or flagged) in one place</t>
+          <t>Development task tracker (this file)</t>
         </is>
       </c>
       <c r="D88" s="13" t="inlineStr">
@@ -3330,7 +3330,7 @@
       <c r="E88" s="16" t="inlineStr"/>
       <c r="F88" s="17" t="inlineStr">
         <is>
-          <t>New openExceptions() in verification.js; returned by GET /applications/:id; rendered as a card at the top of the Documents tab</t>
+          <t>Prepared 2026-09-11, moved to Excel — update statuses as work progresses</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="C89" s="15" t="inlineStr">
         <is>
-          <t>Targeted self-service re-upload — fix exactly one flagged/missing item, no restart</t>
+          <t>Unified 'Action needed' list — every open issue (missing or flagged) in one place</t>
         </is>
       </c>
       <c r="D89" s="13" t="inlineStr">
@@ -3356,7 +3356,7 @@
       <c r="E89" s="16" t="inlineStr"/>
       <c r="F89" s="17" t="inlineStr">
         <is>
-          <t>expectedDocType passed on upload; this is the in-app equivalent of the 'SMS/magic-link' concept — same outcome, no external channel needed since it's already inside the app</t>
+          <t>New openExceptions() in verification.js; returned by GET /applications/:id; rendered as a card at the top of the Documents tab</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>Wrong-file-type caught immediately during a targeted re-upload</t>
+          <t>Targeted self-service re-upload — fix exactly one flagged/missing item, no restart</t>
         </is>
       </c>
       <c r="D90" s="13" t="inlineStr">
@@ -3382,7 +3382,7 @@
       <c r="E90" s="16" t="inlineStr"/>
       <c r="F90" s="17" t="inlineStr">
         <is>
-          <t>New 'Document type' check in verifyDocument() when expectedDocType doesn't match the classified docType</t>
+          <t>expectedDocType passed on upload; this is the in-app equivalent of the 'SMS/magic-link' concept — same outcome, no external channel needed since it's already inside the app</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="C91" s="15" t="inlineStr">
         <is>
-          <t>Document supersede/audit-trail model (current vs. superseded)</t>
+          <t>Wrong-file-type caught immediately during a targeted re-upload</t>
         </is>
       </c>
       <c r="D91" s="13" t="inlineStr">
@@ -3408,7 +3408,7 @@
       <c r="E91" s="16" t="inlineStr"/>
       <c r="F91" s="17" t="inlineStr">
         <is>
-          <t>Document.status field; fixing an item replaces it instead of leaving a duplicate; superseded docs kept for audit, hidden by default behind 'Show document history'</t>
+          <t>New 'Document type' check in verifyDocument() when expectedDocType doesn't match the classified docType</t>
         </is>
       </c>
     </row>
@@ -3423,7 +3423,7 @@
       </c>
       <c r="C92" s="15" t="inlineStr">
         <is>
-          <t>Application status self-heals (Needs Review -&gt; Submitted) once every exception clears</t>
+          <t>Document supersede/audit-trail model (current vs. superseded)</t>
         </is>
       </c>
       <c r="D92" s="13" t="inlineStr">
@@ -3434,7 +3434,7 @@
       <c r="E92" s="16" t="inlineStr"/>
       <c r="F92" s="17" t="inlineStr">
         <is>
-          <t>routes/documents.js — no manual officer action required to un-flag a resolved application</t>
+          <t>Document.status field; fixing an item replaces it instead of leaving a duplicate; superseded docs kept for audit, hidden by default behind 'Show document history'</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="C93" s="15" t="inlineStr">
         <is>
-          <t>Borrower upload endpoint scoped to their own application (auth fix)</t>
+          <t>Application status self-heals (Needs Review -&gt; Submitted) once every exception clears</t>
         </is>
       </c>
       <c r="D93" s="13" t="inlineStr">
@@ -3460,7 +3460,7 @@
       <c r="E93" s="16" t="inlineStr"/>
       <c r="F93" s="17" t="inlineStr">
         <is>
-          <t>POST /documents/:applicationId had no ownership check before today — any authenticated borrower could upload to any applicationId. Now matches the same check already used on GET /applications/:id</t>
+          <t>routes/documents.js — no manual officer action required to un-flag a resolved application</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3475,7 @@
       </c>
       <c r="C94" s="15" t="inlineStr">
         <is>
-          <t>RAG assistant reflects only current, unresolved exceptions</t>
+          <t>Borrower upload endpoint scoped to their own application (auth fix)</t>
         </is>
       </c>
       <c r="D94" s="13" t="inlineStr">
@@ -3486,7 +3486,7 @@
       <c r="E94" s="16" t="inlineStr"/>
       <c r="F94" s="17" t="inlineStr">
         <is>
-          <t>rag.js's applicationStateSummary was reading ALL documents including superseded ones — a resolved issue could be re-surfaced in an answer as if still open. Fixed to use only current documents + the same openExceptions list the UI shows</t>
+          <t>POST /documents/:applicationId had no ownership check before today — any authenticated borrower could upload to any applicationId. Now matches the same check already used on GET /applications/:id</t>
         </is>
       </c>
     </row>
@@ -3501,18 +3501,18 @@
       </c>
       <c r="C95" s="15" t="inlineStr">
         <is>
-          <t>In-browser instant document classification &amp; quality check at upload</t>
+          <t>RAG assistant reflects only current, unresolved exceptions</t>
         </is>
       </c>
       <c r="D95" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E95" s="16" t="inlineStr"/>
       <c r="F95" s="17" t="inlineStr">
         <is>
-          <t>Client-side pre-submission check, before the file is even sent — different from the (built) post-upload flagging</t>
+          <t>rag.js's applicationStateSummary was reading ALL documents including superseded ones — a resolved issue could be re-surfaced in an answer as if still open. Fixed to use only current documents + the same openExceptions list the UI shows</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="C96" s="15" t="inlineStr">
         <is>
-          <t>Pre-submission completeness check (required schedules/pages present)</t>
+          <t>In-browser instant document classification &amp; quality check at upload</t>
         </is>
       </c>
       <c r="D96" s="13" t="inlineStr">
@@ -3538,7 +3538,7 @@
       <c r="E96" s="16" t="inlineStr"/>
       <c r="F96" s="17" t="inlineStr">
         <is>
-          <t>Per document type</t>
+          <t>Client-side pre-submission check, before the file is even sent — different from the (built) post-upload flagging</t>
         </is>
       </c>
     </row>
@@ -3553,7 +3553,7 @@
       </c>
       <c r="C97" s="15" t="inlineStr">
         <is>
-          <t>Blur / glare / legibility detection before accepting an upload</t>
+          <t>Pre-submission completeness check (required schedules/pages present)</t>
         </is>
       </c>
       <c r="D97" s="13" t="inlineStr">
@@ -3564,7 +3564,7 @@
       <c r="E97" s="16" t="inlineStr"/>
       <c r="F97" s="17" t="inlineStr">
         <is>
-          <t>Complements existing confidence-score routing in verification.js</t>
+          <t>Per document type</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3579,7 @@
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>Auto pre-fill of underwriting review fields from extracted data</t>
+          <t>Blur / glare / legibility detection before accepting an upload</t>
         </is>
       </c>
       <c r="D98" s="13" t="inlineStr">
@@ -3590,7 +3590,7 @@
       <c r="E98" s="16" t="inlineStr"/>
       <c r="F98" s="17" t="inlineStr">
         <is>
-          <t>Extraction already produces the data; pre-filling a review form UI is net-new</t>
+          <t>Complements existing confidence-score routing in verification.js</t>
         </is>
       </c>
     </row>
@@ -3600,12 +3600,12 @@
       </c>
       <c r="B99" s="14" t="inlineStr">
         <is>
-          <t>14. Multi-Party &amp; Milestone Tracking (Lending Co-Pilot)</t>
+          <t>13. Real-Time Document Validation &amp; Self-Service Re-Request (DocuSense)</t>
         </is>
       </c>
       <c r="C99" s="15" t="inlineStr">
         <is>
-          <t>Step-by-step milestone tracker UI (Intake -&gt; Doc Verification -&gt; Underwriting -&gt; Closing -&gt; Disbursement)</t>
+          <t>Auto pre-fill of underwriting review fields from extracted data</t>
         </is>
       </c>
       <c r="D99" s="13" t="inlineStr">
@@ -3616,7 +3616,7 @@
       <c r="E99" s="16" t="inlineStr"/>
       <c r="F99" s="17" t="inlineStr">
         <is>
-          <t>New status model, beyond the current submitted/needs-review/approved/rejected enum</t>
+          <t>Extraction already produces the data; pre-filling a review form UI is net-new</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="C100" s="15" t="inlineStr">
         <is>
-          <t>Multi-party checklist — per-owner/signer verification status for business loans</t>
+          <t>Step-by-step milestone tracker UI (Intake -&gt; Doc Verification -&gt; Underwriting -&gt; Closing -&gt; Disbursement)</t>
         </is>
       </c>
       <c r="D100" s="13" t="inlineStr">
@@ -3642,7 +3642,7 @@
       <c r="E100" s="16" t="inlineStr"/>
       <c r="F100" s="17" t="inlineStr">
         <is>
-          <t>Builds on the ownership-disclosure doc type; needs a per-owner sub-record, not just one applicant</t>
+          <t>New status model, beyond the current submitted/needs-review/approved/rejected enum</t>
         </is>
       </c>
     </row>
@@ -3657,7 +3657,7 @@
       </c>
       <c r="C101" s="15" t="inlineStr">
         <is>
-          <t>Shared visibility for all parties on one application</t>
+          <t>Multi-party checklist — per-owner/signer verification status for business loans</t>
         </is>
       </c>
       <c r="D101" s="13" t="inlineStr">
@@ -3668,7 +3668,7 @@
       <c r="E101" s="16" t="inlineStr"/>
       <c r="F101" s="17" t="inlineStr">
         <is>
-          <t>Officer and the single applicant now see the exact same live exception list (built in Section 13's live-exception flow) — what's still missing is MULTIPLE distinct people (co-owners/guarantors) on one application; auth model currently ties an application to one applicant email only</t>
+          <t>Builds on the ownership-disclosure doc type; needs a per-owner sub-record, not just one applicant</t>
         </is>
       </c>
     </row>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C102" s="15" t="inlineStr">
         <is>
-          <t>Core-readiness / entity-name pre-validator earlier in the flow</t>
+          <t>Shared visibility for all parties on one application</t>
         </is>
       </c>
       <c r="D102" s="13" t="inlineStr">
@@ -3694,7 +3694,7 @@
       <c r="E102" s="16" t="inlineStr"/>
       <c r="F102" s="17" t="inlineStr">
         <is>
-          <t>Extends the Section 5 business-name check to run at intake, before final closing</t>
+          <t>Officer and the single applicant now see the exact same live exception list (built in Section 13's live-exception flow) — what's still missing is MULTIPLE distinct people (co-owners/guarantors) on one application; auth model currently ties an application to one applicant email only</t>
         </is>
       </c>
     </row>
@@ -3704,12 +3704,12 @@
       </c>
       <c r="B103" s="14" t="inlineStr">
         <is>
-          <t>15. Predictive Servicing (EarlyCare) — Post-MVP</t>
+          <t>14. Multi-Party &amp; Milestone Tracking (Lending Co-Pilot)</t>
         </is>
       </c>
       <c r="C103" s="15" t="inlineStr">
         <is>
-          <t>Cash-flow dip / pre-delinquency risk detection from transaction history</t>
+          <t>Core-readiness / entity-name pre-validator earlier in the flow</t>
         </is>
       </c>
       <c r="D103" s="13" t="inlineStr">
@@ -3720,7 +3720,7 @@
       <c r="E103" s="16" t="inlineStr"/>
       <c r="F103" s="17" t="inlineStr">
         <is>
-          <t>Different lifecycle stage (servicing, not origination) — needs a transaction-history data model not in the current schema. Recommend as roadmap/vision talking point, not a 4-week build target</t>
+          <t>Extends the Section 5 business-name check to run at intake, before final closing</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3735,7 @@
       </c>
       <c r="C104" s="15" t="inlineStr">
         <is>
-          <t>Self-service grace period / split-payment offers</t>
+          <t>Cash-flow dip / pre-delinquency risk detection from transaction history</t>
         </is>
       </c>
       <c r="D104" s="13" t="inlineStr">
@@ -3746,13 +3746,39 @@
       <c r="E104" s="16" t="inlineStr"/>
       <c r="F104" s="17" t="inlineStr">
         <is>
+          <t>Different lifecycle stage (servicing, not origination) — needs a transaction-history data model not in the current schema. Recommend as roadmap/vision talking point, not a 4-week build target</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="30" customHeight="1">
+      <c r="A105" s="13" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="14" t="inlineStr">
+        <is>
+          <t>15. Predictive Servicing (EarlyCare) — Post-MVP</t>
+        </is>
+      </c>
+      <c r="C105" s="15" t="inlineStr">
+        <is>
+          <t>Self-service grace period / split-payment offers</t>
+        </is>
+      </c>
+      <c r="D105" s="13" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E105" s="16" t="inlineStr"/>
+      <c r="F105" s="17" t="inlineStr">
+        <is>
           <t>Same caveat as above — deprioritize for the MVP</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F104"/>
-  <conditionalFormatting sqref="D2:D104">
+  <autoFilter ref="A1:F105"/>
+  <conditionalFormatting sqref="D2:D105">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$D2="Completed"</formula>
     </cfRule>
@@ -3764,7 +3790,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Completed,In Progress,Not Started"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3778,7 +3804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4597,9 +4623,79 @@
         </is>
       </c>
     </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="13" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>MOCK_AI bypass</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>Mock extraction reproduces the exact planted mismatch for a known seed filename</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>Set MOCK_AI=true, upload jordan-rivera-pay-stub.png.</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>Extraction returns income $4,200 (no real API call); verification flags the same $5,000 vs $4,200 mismatch as the real Claude call would.</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>Confirms the bypass is faithful to real behavior, not just a stub that unblocks the UI — ran this exact case directly against verification.js and got the identical flagged result.</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>Yes — executed directly against verification.js with real inputs (see chat transcript)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>MOCK_AI bypass</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>Unrecognized filename in mock mode degrades gracefully</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>With MOCK_AI=true, upload any file not in the known seed set.</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>Returns docType 'unknown', confidence 0.3 — routes to human review, same as a real illegible document, instead of throwing.</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>So testing with an arbitrary file doesn't crash the upload flow while mock mode is on.</t>
+        </is>
+      </c>
+      <c r="G25" s="18" t="inlineStr">
+        <is>
+          <t>Yes — executed directly against verification.js with real inputs (see chat transcript)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G23"/>
-  <conditionalFormatting sqref="G2:G23">
+  <autoFilter ref="A1:G25"/>
+  <conditionalFormatting sqref="G2:G25">
     <cfRule type="expression" priority="1" dxfId="3">
       <formula>LEFT($G2,3)="Yes"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add Indian-named seed borrowers with real logins
- Priya Nair (already existed as an application-only record, no login)
  now has a real borrower login
- Renamed the "Marcus Webb" auto-loan record to Arjun Mehta with a real
  login too — safe rename, that name wasn't referenced anywhere outside
  the two seed scripts
- Jordan Rivera and Dana Whitfield left as-is (flagship scenarios,
  deeply referenced in DEMO_SCRIPT.md and test-questions.md)
- Going forward: use Indian names for any new seed/test data

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LoanLensAI_Development_Task_Tracker.xlsx
+++ b/docs/LoanLensAI_Development_Task_Tracker.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenarios" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$F$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$F$106</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test Scenarios'!$A$1:$G$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -700,15 +700,15 @@
     </row>
     <row r="13">
       <c r="A13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="D13" s="7">
@@ -757,15 +757,15 @@
         </is>
       </c>
       <c r="B18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A18,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A18,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A18,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A18,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A18,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A18,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E18" s="10">
@@ -780,15 +780,15 @@
         </is>
       </c>
       <c r="B19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A19,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A19,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A19,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A19,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A19,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A19,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E19" s="10">
@@ -803,15 +803,15 @@
         </is>
       </c>
       <c r="B20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A20,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A20,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A20,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A20,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A20,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A20,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E20" s="10">
@@ -826,15 +826,15 @@
         </is>
       </c>
       <c r="B21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A21,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A21,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A21,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A21,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A21,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A21,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E21" s="10">
@@ -849,15 +849,15 @@
         </is>
       </c>
       <c r="B22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A22,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A22,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A22,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A22,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A22,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A22,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E22" s="10">
@@ -872,15 +872,15 @@
         </is>
       </c>
       <c r="B23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A23,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A23,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A23,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A23,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A23,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A23,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E23" s="10">
@@ -895,15 +895,15 @@
         </is>
       </c>
       <c r="B24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A24,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A24,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A24,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A24,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A24,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A24,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E24" s="10">
@@ -918,15 +918,15 @@
         </is>
       </c>
       <c r="B25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A25,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A25,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A25,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A25,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A25,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A25,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E25" s="10">
@@ -941,15 +941,15 @@
         </is>
       </c>
       <c r="B26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A26,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A26,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A26,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A26,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A26,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A26,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E26" s="10">
@@ -964,15 +964,15 @@
         </is>
       </c>
       <c r="B27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A27,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A27,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A27,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A27,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A27,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A27,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E27" s="10">
@@ -987,15 +987,15 @@
         </is>
       </c>
       <c r="B28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A28,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A28,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A28,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A28,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A28,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A28,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E28" s="10">
@@ -1010,15 +1010,15 @@
         </is>
       </c>
       <c r="B29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A29,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A29,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A29,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A29,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A29,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A29,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E29" s="10">
@@ -1033,15 +1033,15 @@
         </is>
       </c>
       <c r="B30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A30,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A30,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A30,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A30,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A30,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A30,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E30" s="10">
@@ -1056,15 +1056,15 @@
         </is>
       </c>
       <c r="B31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A31,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A31,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A31,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A31,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A31,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A31,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E31" s="10">
@@ -1079,15 +1079,15 @@
         </is>
       </c>
       <c r="B32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A32,Tasks!$D$2:$D$105,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A32,Tasks!$D$2:$D$106,"Completed")</f>
         <v/>
       </c>
       <c r="C32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A32,Tasks!$D$2:$D$105,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A32,Tasks!$D$2:$D$106,"In Progress")</f>
         <v/>
       </c>
       <c r="D32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$105,$A32,Tasks!$D$2:$D$105,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$106,$A32,Tasks!$D$2:$D$106,"Not Started")</f>
         <v/>
       </c>
       <c r="E32" s="10">
@@ -1109,7 +1109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2900,23 +2900,23 @@
       </c>
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t>9. WhatsApp Integration</t>
+          <t>8. Synthetic Demo Data</t>
         </is>
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>Meta developer app + free sandbox test number</t>
+          <t>Indian-named seed borrowers with real logins (Priya Nair, Arjun Mehta)</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E71" s="16" t="inlineStr"/>
       <c r="F71" s="17" t="inlineStr">
         <is>
-          <t>Self-serve, free, no leadership approval needed for the demo</t>
+          <t>Priya Nair already existed as an application-only record (no login); Arjun Mehta replaces the former 'Marcus Webb' auto-loan record (safe — that name wasn't referenced in DEMO_SCRIPT.md or test-questions.md). Standing preference going forward: use Indian names for any new seed/test data added</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>Webhook endpoint to receive inbound WhatsApp messages</t>
+          <t>Meta developer app + free sandbox test number</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr">
@@ -2940,7 +2940,11 @@
         </is>
       </c>
       <c r="E72" s="16" t="inlineStr"/>
-      <c r="F72" s="17" t="inlineStr"/>
+      <c r="F72" s="17" t="inlineStr">
+        <is>
+          <t>Self-serve, free, no leadership approval needed for the demo</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="13" t="n">
@@ -2953,7 +2957,7 @@
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>Route inbound messages into the existing RAG assistant</t>
+          <t>Webhook endpoint to receive inbound WhatsApp messages</t>
         </is>
       </c>
       <c r="D73" s="13" t="inlineStr">
@@ -2962,11 +2966,7 @@
         </is>
       </c>
       <c r="E73" s="16" t="inlineStr"/>
-      <c r="F73" s="17" t="inlineStr">
-        <is>
-          <t>Can reuse services/rag.js — answerQuestion()</t>
-        </is>
-      </c>
+      <c r="F73" s="17" t="inlineStr"/>
     </row>
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="13" t="n">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>Outbound reply via WhatsApp Cloud API</t>
+          <t>Route inbound messages into the existing RAG assistant</t>
         </is>
       </c>
       <c r="D74" s="13" t="inlineStr">
@@ -2988,7 +2988,11 @@
         </is>
       </c>
       <c r="E74" s="16" t="inlineStr"/>
-      <c r="F74" s="17" t="inlineStr"/>
+      <c r="F74" s="17" t="inlineStr">
+        <is>
+          <t>Can reuse services/rag.js — answerQuestion()</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="13" t="n">
@@ -3001,7 +3005,7 @@
       </c>
       <c r="C75" s="15" t="inlineStr">
         <is>
-          <t>Production Meta Business verification</t>
+          <t>Outbound reply via WhatsApp Cloud API</t>
         </is>
       </c>
       <c r="D75" s="13" t="inlineStr">
@@ -3010,11 +3014,7 @@
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr"/>
-      <c r="F75" s="17" t="inlineStr">
-        <is>
-          <t>Only needed post-demo, for a real bank pilot — not for the MVP</t>
-        </is>
-      </c>
+      <c r="F75" s="17" t="inlineStr"/>
     </row>
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="13" t="n">
@@ -3022,23 +3022,23 @@
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>10. Hosting &amp; Deployment</t>
+          <t>9. WhatsApp Integration</t>
         </is>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>Render Blueprint configuration</t>
+          <t>Production Meta Business verification</t>
         </is>
       </c>
       <c r="D76" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E76" s="16" t="inlineStr"/>
       <c r="F76" s="17" t="inlineStr">
         <is>
-          <t>render.yaml — backend web service + frontend static site</t>
+          <t>Only needed post-demo, for a real bank pilot — not for the MVP</t>
         </is>
       </c>
     </row>
@@ -3053,18 +3053,18 @@
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>Backend deployed &amp; health-checked on Render</t>
+          <t>Render Blueprint configuration</t>
         </is>
       </c>
       <c r="D77" s="13" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E77" s="16" t="inlineStr"/>
       <c r="F77" s="17" t="inlineStr">
         <is>
-          <t>Confirm live and reachable before demo day (/health)</t>
+          <t>render.yaml — backend web service + frontend static site</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>Frontend deployed as Render static site</t>
+          <t>Backend deployed &amp; health-checked on Render</t>
         </is>
       </c>
       <c r="D78" s="13" t="inlineStr">
@@ -3090,7 +3090,7 @@
       <c r="E78" s="16" t="inlineStr"/>
       <c r="F78" s="17" t="inlineStr">
         <is>
-          <t>Confirm Expo web export + rewrite rule are working</t>
+          <t>Confirm live and reachable before demo day (/health)</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="C79" s="15" t="inlineStr">
         <is>
-          <t>MongoDB Atlas cluster provisioned (M0 free tier)</t>
+          <t>Frontend deployed as Render static site</t>
         </is>
       </c>
       <c r="D79" s="13" t="inlineStr">
@@ -3116,7 +3116,7 @@
       <c r="E79" s="16" t="inlineStr"/>
       <c r="F79" s="17" t="inlineStr">
         <is>
-          <t>Confirm connection string + Network Access 0.0.0.0/0 are set</t>
+          <t>Confirm Expo web export + rewrite rule are working</t>
         </is>
       </c>
     </row>
@@ -3131,18 +3131,18 @@
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>One-shot /admin/reset endpoint for pre-demo data reset</t>
+          <t>MongoDB Atlas cluster provisioned (M0 free tier)</t>
         </is>
       </c>
       <c r="D80" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E80" s="16" t="inlineStr"/>
       <c r="F80" s="17" t="inlineStr">
         <is>
-          <t>routes/admin.js — seeds + re-indexes policies in one call</t>
+          <t>Confirm connection string + Network Access 0.0.0.0/0 are set</t>
         </is>
       </c>
     </row>
@@ -3152,12 +3152,12 @@
       </c>
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>11. Testing &amp; QA</t>
+          <t>10. Hosting &amp; Deployment</t>
         </is>
       </c>
       <c r="C81" s="15" t="inlineStr">
         <is>
-          <t>Manual acceptance test question bank</t>
+          <t>One-shot /admin/reset endpoint for pre-demo data reset</t>
         </is>
       </c>
       <c r="D81" s="13" t="inlineStr">
@@ -3168,7 +3168,7 @@
       <c r="E81" s="16" t="inlineStr"/>
       <c r="F81" s="17" t="inlineStr">
         <is>
-          <t>23 questions across consumer + small-business scenarios</t>
+          <t>routes/admin.js — seeds + re-indexes policies in one call</t>
         </is>
       </c>
     </row>
@@ -3183,16 +3183,20 @@
       </c>
       <c r="C82" s="15" t="inlineStr">
         <is>
-          <t>Automated unit/integration tests</t>
+          <t>Manual acceptance test question bank</t>
         </is>
       </c>
       <c r="D82" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E82" s="16" t="inlineStr"/>
-      <c r="F82" s="17" t="inlineStr"/>
+      <c r="F82" s="17" t="inlineStr">
+        <is>
+          <t>23 questions across consumer + small-business scenarios</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="13" t="n">
@@ -3205,7 +3209,7 @@
       </c>
       <c r="C83" s="15" t="inlineStr">
         <is>
-          <t>End-to-end demo rehearsal (full run-through, timed)</t>
+          <t>Automated unit/integration tests</t>
         </is>
       </c>
       <c r="D83" s="13" t="inlineStr">
@@ -3214,11 +3218,7 @@
         </is>
       </c>
       <c r="E83" s="16" t="inlineStr"/>
-      <c r="F83" s="17" t="inlineStr">
-        <is>
-          <t>Schedule before presentation day</t>
-        </is>
-      </c>
+      <c r="F83" s="17" t="inlineStr"/>
     </row>
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="13" t="n">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Cross-browser / device check (Expo web export)</t>
+          <t>End-to-end demo rehearsal (full run-through, timed)</t>
         </is>
       </c>
       <c r="D84" s="13" t="inlineStr">
@@ -3240,7 +3240,11 @@
         </is>
       </c>
       <c r="E84" s="16" t="inlineStr"/>
-      <c r="F84" s="17" t="inlineStr"/>
+      <c r="F84" s="17" t="inlineStr">
+        <is>
+          <t>Schedule before presentation day</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="13" t="n">
@@ -3248,17 +3252,17 @@
       </c>
       <c r="B85" s="14" t="inlineStr">
         <is>
-          <t>12. Documentation</t>
+          <t>11. Testing &amp; QA</t>
         </is>
       </c>
       <c r="C85" s="15" t="inlineStr">
         <is>
-          <t>README (quick start, architecture, deploy steps)</t>
+          <t>Cross-browser / device check (Expo web export)</t>
         </is>
       </c>
       <c r="D85" s="13" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E85" s="16" t="inlineStr"/>
@@ -3275,7 +3279,7 @@
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>ROADMAP.md (phased build plan)</t>
+          <t>README (quick start, architecture, deploy steps)</t>
         </is>
       </c>
       <c r="D86" s="13" t="inlineStr">
@@ -3297,7 +3301,7 @@
       </c>
       <c r="C87" s="15" t="inlineStr">
         <is>
-          <t>DEMO_SCRIPT.md (3-minute walkthrough)</t>
+          <t>ROADMAP.md (phased build plan)</t>
         </is>
       </c>
       <c r="D87" s="13" t="inlineStr">
@@ -3319,7 +3323,7 @@
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Development task tracker (this file)</t>
+          <t>DEMO_SCRIPT.md (3-minute walkthrough)</t>
         </is>
       </c>
       <c r="D88" s="13" t="inlineStr">
@@ -3328,11 +3332,7 @@
         </is>
       </c>
       <c r="E88" s="16" t="inlineStr"/>
-      <c r="F88" s="17" t="inlineStr">
-        <is>
-          <t>Prepared 2026-09-11, moved to Excel — update statuses as work progresses</t>
-        </is>
-      </c>
+      <c r="F88" s="17" t="inlineStr"/>
     </row>
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="13" t="n">
@@ -3340,12 +3340,12 @@
       </c>
       <c r="B89" s="14" t="inlineStr">
         <is>
-          <t>13. Real-Time Document Validation &amp; Self-Service Re-Request (DocuSense)</t>
+          <t>12. Documentation</t>
         </is>
       </c>
       <c r="C89" s="15" t="inlineStr">
         <is>
-          <t>Unified 'Action needed' list — every open issue (missing or flagged) in one place</t>
+          <t>Development task tracker (this file)</t>
         </is>
       </c>
       <c r="D89" s="13" t="inlineStr">
@@ -3356,7 +3356,7 @@
       <c r="E89" s="16" t="inlineStr"/>
       <c r="F89" s="17" t="inlineStr">
         <is>
-          <t>New openExceptions() in verification.js; returned by GET /applications/:id; rendered as a card at the top of the Documents tab</t>
+          <t>Prepared 2026-09-11, moved to Excel — update statuses as work progresses</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>Targeted self-service re-upload — fix exactly one flagged/missing item, no restart</t>
+          <t>Unified 'Action needed' list — every open issue (missing or flagged) in one place</t>
         </is>
       </c>
       <c r="D90" s="13" t="inlineStr">
@@ -3382,7 +3382,7 @@
       <c r="E90" s="16" t="inlineStr"/>
       <c r="F90" s="17" t="inlineStr">
         <is>
-          <t>expectedDocType passed on upload; this is the in-app equivalent of the 'SMS/magic-link' concept — same outcome, no external channel needed since it's already inside the app</t>
+          <t>New openExceptions() in verification.js; returned by GET /applications/:id; rendered as a card at the top of the Documents tab</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="C91" s="15" t="inlineStr">
         <is>
-          <t>Wrong-file-type caught immediately during a targeted re-upload</t>
+          <t>Targeted self-service re-upload — fix exactly one flagged/missing item, no restart</t>
         </is>
       </c>
       <c r="D91" s="13" t="inlineStr">
@@ -3408,7 +3408,7 @@
       <c r="E91" s="16" t="inlineStr"/>
       <c r="F91" s="17" t="inlineStr">
         <is>
-          <t>New 'Document type' check in verifyDocument() when expectedDocType doesn't match the classified docType</t>
+          <t>expectedDocType passed on upload; this is the in-app equivalent of the 'SMS/magic-link' concept — same outcome, no external channel needed since it's already inside the app</t>
         </is>
       </c>
     </row>
@@ -3423,7 +3423,7 @@
       </c>
       <c r="C92" s="15" t="inlineStr">
         <is>
-          <t>Document supersede/audit-trail model (current vs. superseded)</t>
+          <t>Wrong-file-type caught immediately during a targeted re-upload</t>
         </is>
       </c>
       <c r="D92" s="13" t="inlineStr">
@@ -3434,7 +3434,7 @@
       <c r="E92" s="16" t="inlineStr"/>
       <c r="F92" s="17" t="inlineStr">
         <is>
-          <t>Document.status field; fixing an item replaces it instead of leaving a duplicate; superseded docs kept for audit, hidden by default behind 'Show document history'</t>
+          <t>New 'Document type' check in verifyDocument() when expectedDocType doesn't match the classified docType</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="C93" s="15" t="inlineStr">
         <is>
-          <t>Application status self-heals (Needs Review -&gt; Submitted) once every exception clears</t>
+          <t>Document supersede/audit-trail model (current vs. superseded)</t>
         </is>
       </c>
       <c r="D93" s="13" t="inlineStr">
@@ -3460,7 +3460,7 @@
       <c r="E93" s="16" t="inlineStr"/>
       <c r="F93" s="17" t="inlineStr">
         <is>
-          <t>routes/documents.js — no manual officer action required to un-flag a resolved application</t>
+          <t>Document.status field; fixing an item replaces it instead of leaving a duplicate; superseded docs kept for audit, hidden by default behind 'Show document history'</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3475,7 @@
       </c>
       <c r="C94" s="15" t="inlineStr">
         <is>
-          <t>Borrower upload endpoint scoped to their own application (auth fix)</t>
+          <t>Application status self-heals (Needs Review -&gt; Submitted) once every exception clears</t>
         </is>
       </c>
       <c r="D94" s="13" t="inlineStr">
@@ -3486,7 +3486,7 @@
       <c r="E94" s="16" t="inlineStr"/>
       <c r="F94" s="17" t="inlineStr">
         <is>
-          <t>POST /documents/:applicationId had no ownership check before today — any authenticated borrower could upload to any applicationId. Now matches the same check already used on GET /applications/:id</t>
+          <t>routes/documents.js — no manual officer action required to un-flag a resolved application</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="C95" s="15" t="inlineStr">
         <is>
-          <t>RAG assistant reflects only current, unresolved exceptions</t>
+          <t>Borrower upload endpoint scoped to their own application (auth fix)</t>
         </is>
       </c>
       <c r="D95" s="13" t="inlineStr">
@@ -3512,7 +3512,7 @@
       <c r="E95" s="16" t="inlineStr"/>
       <c r="F95" s="17" t="inlineStr">
         <is>
-          <t>rag.js's applicationStateSummary was reading ALL documents including superseded ones — a resolved issue could be re-surfaced in an answer as if still open. Fixed to use only current documents + the same openExceptions list the UI shows</t>
+          <t>POST /documents/:applicationId had no ownership check before today — any authenticated borrower could upload to any applicationId. Now matches the same check already used on GET /applications/:id</t>
         </is>
       </c>
     </row>
@@ -3527,18 +3527,18 @@
       </c>
       <c r="C96" s="15" t="inlineStr">
         <is>
-          <t>In-browser instant document classification &amp; quality check at upload</t>
+          <t>RAG assistant reflects only current, unresolved exceptions</t>
         </is>
       </c>
       <c r="D96" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E96" s="16" t="inlineStr"/>
       <c r="F96" s="17" t="inlineStr">
         <is>
-          <t>Client-side pre-submission check, before the file is even sent — different from the (built) post-upload flagging</t>
+          <t>rag.js's applicationStateSummary was reading ALL documents including superseded ones — a resolved issue could be re-surfaced in an answer as if still open. Fixed to use only current documents + the same openExceptions list the UI shows</t>
         </is>
       </c>
     </row>
@@ -3553,7 +3553,7 @@
       </c>
       <c r="C97" s="15" t="inlineStr">
         <is>
-          <t>Pre-submission completeness check (required schedules/pages present)</t>
+          <t>In-browser instant document classification &amp; quality check at upload</t>
         </is>
       </c>
       <c r="D97" s="13" t="inlineStr">
@@ -3564,7 +3564,7 @@
       <c r="E97" s="16" t="inlineStr"/>
       <c r="F97" s="17" t="inlineStr">
         <is>
-          <t>Per document type</t>
+          <t>Client-side pre-submission check, before the file is even sent — different from the (built) post-upload flagging</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3579,7 @@
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>Blur / glare / legibility detection before accepting an upload</t>
+          <t>Pre-submission completeness check (required schedules/pages present)</t>
         </is>
       </c>
       <c r="D98" s="13" t="inlineStr">
@@ -3590,7 +3590,7 @@
       <c r="E98" s="16" t="inlineStr"/>
       <c r="F98" s="17" t="inlineStr">
         <is>
-          <t>Complements existing confidence-score routing in verification.js</t>
+          <t>Per document type</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="C99" s="15" t="inlineStr">
         <is>
-          <t>Auto pre-fill of underwriting review fields from extracted data</t>
+          <t>Blur / glare / legibility detection before accepting an upload</t>
         </is>
       </c>
       <c r="D99" s="13" t="inlineStr">
@@ -3616,7 +3616,7 @@
       <c r="E99" s="16" t="inlineStr"/>
       <c r="F99" s="17" t="inlineStr">
         <is>
-          <t>Extraction already produces the data; pre-filling a review form UI is net-new</t>
+          <t>Complements existing confidence-score routing in verification.js</t>
         </is>
       </c>
     </row>
@@ -3626,12 +3626,12 @@
       </c>
       <c r="B100" s="14" t="inlineStr">
         <is>
-          <t>14. Multi-Party &amp; Milestone Tracking (Lending Co-Pilot)</t>
+          <t>13. Real-Time Document Validation &amp; Self-Service Re-Request (DocuSense)</t>
         </is>
       </c>
       <c r="C100" s="15" t="inlineStr">
         <is>
-          <t>Step-by-step milestone tracker UI (Intake -&gt; Doc Verification -&gt; Underwriting -&gt; Closing -&gt; Disbursement)</t>
+          <t>Auto pre-fill of underwriting review fields from extracted data</t>
         </is>
       </c>
       <c r="D100" s="13" t="inlineStr">
@@ -3642,7 +3642,7 @@
       <c r="E100" s="16" t="inlineStr"/>
       <c r="F100" s="17" t="inlineStr">
         <is>
-          <t>New status model, beyond the current submitted/needs-review/approved/rejected enum</t>
+          <t>Extraction already produces the data; pre-filling a review form UI is net-new</t>
         </is>
       </c>
     </row>
@@ -3657,7 +3657,7 @@
       </c>
       <c r="C101" s="15" t="inlineStr">
         <is>
-          <t>Multi-party checklist — per-owner/signer verification status for business loans</t>
+          <t>Step-by-step milestone tracker UI (Intake -&gt; Doc Verification -&gt; Underwriting -&gt; Closing -&gt; Disbursement)</t>
         </is>
       </c>
       <c r="D101" s="13" t="inlineStr">
@@ -3668,7 +3668,7 @@
       <c r="E101" s="16" t="inlineStr"/>
       <c r="F101" s="17" t="inlineStr">
         <is>
-          <t>Builds on the ownership-disclosure doc type; needs a per-owner sub-record, not just one applicant</t>
+          <t>New status model, beyond the current submitted/needs-review/approved/rejected enum</t>
         </is>
       </c>
     </row>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C102" s="15" t="inlineStr">
         <is>
-          <t>Shared visibility for all parties on one application</t>
+          <t>Multi-party checklist — per-owner/signer verification status for business loans</t>
         </is>
       </c>
       <c r="D102" s="13" t="inlineStr">
@@ -3694,7 +3694,7 @@
       <c r="E102" s="16" t="inlineStr"/>
       <c r="F102" s="17" t="inlineStr">
         <is>
-          <t>Officer and the single applicant now see the exact same live exception list (built in Section 13's live-exception flow) — what's still missing is MULTIPLE distinct people (co-owners/guarantors) on one application; auth model currently ties an application to one applicant email only</t>
+          <t>Builds on the ownership-disclosure doc type; needs a per-owner sub-record, not just one applicant</t>
         </is>
       </c>
     </row>
@@ -3709,7 +3709,7 @@
       </c>
       <c r="C103" s="15" t="inlineStr">
         <is>
-          <t>Core-readiness / entity-name pre-validator earlier in the flow</t>
+          <t>Shared visibility for all parties on one application</t>
         </is>
       </c>
       <c r="D103" s="13" t="inlineStr">
@@ -3720,7 +3720,7 @@
       <c r="E103" s="16" t="inlineStr"/>
       <c r="F103" s="17" t="inlineStr">
         <is>
-          <t>Extends the Section 5 business-name check to run at intake, before final closing</t>
+          <t>Officer and the single applicant now see the exact same live exception list (built in Section 13's live-exception flow) — what's still missing is MULTIPLE distinct people (co-owners/guarantors) on one application; auth model currently ties an application to one applicant email only</t>
         </is>
       </c>
     </row>
@@ -3730,12 +3730,12 @@
       </c>
       <c r="B104" s="14" t="inlineStr">
         <is>
-          <t>15. Predictive Servicing (EarlyCare) — Post-MVP</t>
+          <t>14. Multi-Party &amp; Milestone Tracking (Lending Co-Pilot)</t>
         </is>
       </c>
       <c r="C104" s="15" t="inlineStr">
         <is>
-          <t>Cash-flow dip / pre-delinquency risk detection from transaction history</t>
+          <t>Core-readiness / entity-name pre-validator earlier in the flow</t>
         </is>
       </c>
       <c r="D104" s="13" t="inlineStr">
@@ -3746,7 +3746,7 @@
       <c r="E104" s="16" t="inlineStr"/>
       <c r="F104" s="17" t="inlineStr">
         <is>
-          <t>Different lifecycle stage (servicing, not origination) — needs a transaction-history data model not in the current schema. Recommend as roadmap/vision talking point, not a 4-week build target</t>
+          <t>Extends the Section 5 business-name check to run at intake, before final closing</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="C105" s="15" t="inlineStr">
         <is>
-          <t>Self-service grace period / split-payment offers</t>
+          <t>Cash-flow dip / pre-delinquency risk detection from transaction history</t>
         </is>
       </c>
       <c r="D105" s="13" t="inlineStr">
@@ -3772,13 +3772,39 @@
       <c r="E105" s="16" t="inlineStr"/>
       <c r="F105" s="17" t="inlineStr">
         <is>
+          <t>Different lifecycle stage (servicing, not origination) — needs a transaction-history data model not in the current schema. Recommend as roadmap/vision talking point, not a 4-week build target</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="30" customHeight="1">
+      <c r="A106" s="13" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="14" t="inlineStr">
+        <is>
+          <t>15. Predictive Servicing (EarlyCare) — Post-MVP</t>
+        </is>
+      </c>
+      <c r="C106" s="15" t="inlineStr">
+        <is>
+          <t>Self-service grace period / split-payment offers</t>
+        </is>
+      </c>
+      <c r="D106" s="13" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E106" s="16" t="inlineStr"/>
+      <c r="F106" s="17" t="inlineStr">
+        <is>
           <t>Same caveat as above — deprioritize for the MVP</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F105"/>
-  <conditionalFormatting sqref="D2:D105">
+  <autoFilter ref="A1:F106"/>
+  <conditionalFormatting sqref="D2:D106">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$D2="Completed"</formula>
     </cfRule>
@@ -3790,7 +3816,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Completed,In Progress,Not Started"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs: Truth Engine architecture section + tracker sections 16-17
Documents the 4-layer document-truth framework: Layers 2 (statutory
math) and 3 (cross-document) are built and shipped; Layers 1 (digital
forensics) and 4 (external grounding) are explicitly roadmap, needing
a funded vendor relationship rather than more engineering time.

Tracker: marks the 4 checks built this session as Completed under
Section 5, and adds two new sections — 16 (forensics/external
verification, needs API keys + funding) and 17 (KYC/address/credit,
mixed free vs. funded) — so the funding-dependent items are visible
and don't get silently conflated with "not built yet, just needs
more of our own time."

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LoanLensAI_Development_Task_Tracker.xlsx
+++ b/docs/LoanLensAI_Development_Task_Tracker.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -634,6 +634,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -655,6 +656,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
@@ -669,6 +671,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -700,15 +703,15 @@
     </row>
     <row r="13">
       <c r="A13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="D13" s="7">
@@ -716,6 +719,8 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
@@ -757,15 +762,15 @@
         </is>
       </c>
       <c r="B18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A18,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A18,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A18,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A18,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A18,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A18,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E18" s="10">
@@ -780,15 +785,15 @@
         </is>
       </c>
       <c r="B19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A19,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A19,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A19,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A19,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A19,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A19,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E19" s="10">
@@ -803,15 +808,15 @@
         </is>
       </c>
       <c r="B20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A20,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A20,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A20,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A20,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A20,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A20,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E20" s="10">
@@ -826,15 +831,15 @@
         </is>
       </c>
       <c r="B21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A21,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A21,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A21,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A21,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A21,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A21,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E21" s="10">
@@ -849,15 +854,15 @@
         </is>
       </c>
       <c r="B22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A22,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A22,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A22,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A22,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A22,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A22,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E22" s="10">
@@ -872,15 +877,15 @@
         </is>
       </c>
       <c r="B23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A23,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A23,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A23,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A23,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A23,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A23,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E23" s="10">
@@ -895,15 +900,15 @@
         </is>
       </c>
       <c r="B24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A24,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A24,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A24,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A24,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A24,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A24,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E24" s="10">
@@ -918,15 +923,15 @@
         </is>
       </c>
       <c r="B25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A25,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A25,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A25,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A25,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A25,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A25,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E25" s="10">
@@ -941,15 +946,15 @@
         </is>
       </c>
       <c r="B26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A26,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A26,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A26,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A26,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A26,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A26,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E26" s="10">
@@ -964,15 +969,15 @@
         </is>
       </c>
       <c r="B27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A27,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A27,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A27,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A27,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A27,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A27,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E27" s="10">
@@ -987,15 +992,15 @@
         </is>
       </c>
       <c r="B28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A28,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A28,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A28,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A28,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A28,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A28,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E28" s="10">
@@ -1010,15 +1015,15 @@
         </is>
       </c>
       <c r="B29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A29,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A29,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A29,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A29,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A29,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A29,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E29" s="10">
@@ -1033,15 +1038,15 @@
         </is>
       </c>
       <c r="B30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A30,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A30,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A30,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A30,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A30,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A30,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E30" s="10">
@@ -1056,15 +1061,15 @@
         </is>
       </c>
       <c r="B31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A31,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A31,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A31,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A31,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A31,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A31,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E31" s="10">
@@ -1079,19 +1084,65 @@
         </is>
       </c>
       <c r="B32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A32,Tasks!$D$2:$D$118,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A32,Tasks!$D$2:$D$133,"Completed")</f>
         <v/>
       </c>
       <c r="C32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A32,Tasks!$D$2:$D$118,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A32,Tasks!$D$2:$D$133,"In Progress")</f>
         <v/>
       </c>
       <c r="D32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$118,$A32,Tasks!$D$2:$D$118,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A32,Tasks!$D$2:$D$133,"Not Started")</f>
         <v/>
       </c>
       <c r="E32" s="10">
         <f>SUM(B32:D32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>16. Document Authenticity — Digital Forensics &amp; Direct-Source Verification</t>
+        </is>
+      </c>
+      <c r="B33">
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A33,Tasks!$D$2:$D$133,"Completed")</f>
+        <v/>
+      </c>
+      <c r="C33">
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A33,Tasks!$D$2:$D$133,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="D33">
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A33,Tasks!$D$2:$D$133,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="E33">
+        <f>SUM(B33:D33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>17. Identity, Address &amp; Credit Verification (KYC / Underwriting)</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A34,Tasks!$D$2:$D$133,"Completed")</f>
+        <v/>
+      </c>
+      <c r="C34">
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A34,Tasks!$D$2:$D$133,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="D34">
+        <f>COUNTIFS(Tasks!$B$2:$B$133,$A34,Tasks!$D$2:$D$133,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="E34">
+        <f>SUM(B34:D34)</f>
         <v/>
       </c>
     </row>
@@ -1109,7 +1160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F118"/>
+  <dimension ref="A1:F133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4111,6 +4162,381 @@
       <c r="F118" s="17" t="inlineStr">
         <is>
           <t>Same caveat as above — deprioritize for the MVP</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>5. Cross-Verification Engine</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Cross-document check: bank statement deposit vs. pay stub net pay (amount + employer-name match)</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>backend/src/services/verification.js — crossDocumentChecks()/withCrossDocumentChecks(); catches an inflated pay stub not backed by a real deposit</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>5. Cross-Verification Engine</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Statutory payroll-math check: Social Security (6.2%) &amp; Medicare (1.45%) withholding vs. gross pay</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>backend/src/services/verification.js; flat federal rates, not income-tax brackets (deliberately not modeled — see Section 16 note)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>5. Cross-Verification Engine</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Year-to-date gross consistency check (YTD gross ÷ pay period # vs. current period gross)</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>backend/src/services/verification.js; pay stub images regenerated to show YTD gross + period #</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>5. Cross-Verification Engine</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Ownership percentage sanity bound (0-100%)</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>backend/src/services/verification.js; single-doc-per-application model limits this to a bounds check, not a multi-owner sum-to-100% check</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>5. Cross-Verification Engine</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Personal financial statement vs. bank statement cash-on-hand cross-check</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Same buildable pattern as the completed pay-stub/bank-statement check above — no vendor needed, just not yet prioritized</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>16. Document Authenticity — Digital Forensics &amp; Direct-Source Verification</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>PDF metadata / edit-history forensics</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>No vendor cost, but our demo docs are images (no metadata to inspect); even on real PDFs this is easily defeated by re-export/screenshot — low reliability even in production</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>16. Document Authenticity — Digital Forensics &amp; Direct-Source Verification</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Font/glyph and template-mismatch detection</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Needs a reference library of genuine payroll-provider templates (ADP/Gusto/Paychex) — a real computer-vision project, out of hackathon scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>16. Document Authenticity — Digital Forensics &amp; Direct-Source Verification</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Error Level Analysis (ELA) for spliced/edited images</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Free to build (no vendor), but only detects JPEG recompression artifacts — has no effect on our PNG uploads; revisit if real photographed/scanned uploads are supported</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>16. Document Authenticity — Digital Forensics &amp; Direct-Source Verification</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Identity verification (IDV) for driver's license / government ID</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>NEEDS REAL-TIME API KEY + FUNDING — vendor options: Persona, Onfido, Jumio, ID.me (liveness + barcode/MRZ check)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>16. Document Authenticity — Digital Forensics &amp; Direct-Source Verification</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>IRS tax transcript verification (Form 4506-C / IVES) for business tax returns</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>NEEDS FUNDING — requires becoming an approved IVES participant; not obtainable via a simple developer API key sign-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>16. Document Authenticity — Digital Forensics &amp; Direct-Source Verification</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Business registry / EIN verification (Secretary of State lookup)</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>NEEDS REAL-TIME API KEY + FUNDING — vendor option: Middesk (most state registries have no free structured API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>16. Document Authenticity — Digital Forensics &amp; Direct-Source Verification</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Direct-from-source payroll verification (bypass documents entirely)</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>NEEDS REAL-TIME API KEY + FUNDING — vendor options: Argyle, Pinwheel, Plaid Income; this is the actual production-grade fix — uploaded documents become an optional fallback, not the source of truth</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>17. Identity, Address &amp; Credit Verification (KYC / Underwriting)</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>OFAC sanctions / PEP screening for beneficial owners</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>FREE — U.S. Treasury OFAC SDN list is a public, free, downloadable dataset; no paid vendor required to build a basic screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>17. Identity, Address &amp; Credit Verification (KYC / Underwriting)</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Address verification (standardization + deliverability)</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>FREE TIER AVAILABLE — USPS Web Tools API has a no-cost tier suitable for this use case</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>17. Identity, Address &amp; Credit Verification (KYC / Underwriting)</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Credit bureau pull / existing-loan (trade line) check</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>NEEDS FUNDING — real bureau access (Equifax/Experian/TransUnion) requires a licensed FCRA "permissible purpose" relationship, not just an API key; soft-pull aggregators (Array, Bloom Credit, MeridianLink) are the realistic funded path</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update task tracker with underwriter workflow, proposal gaps and policy work
- New sections 18 (decision / underwriter workflow), 19 (proposal gaps),
  20 (policy documents and policy page): 56 new tasks
- Session work recorded as completed (verification checklist, page URLs,
  progress / action-needed pages, chat navigation)
- Corrected statuses on automated tests and the milestone tracker
- Filter, status dropdown and colours now cover every row (they stopped at 118)
- 11 new test scenarios and a "Proposal vs Built" sheet

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LoanLensAI_Development_Task_Tracker.xlsx
+++ b/docs/LoanLensAI_Development_Task_Tracker.xlsx
@@ -10,10 +10,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenarios" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proposal vs Built" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$F$118</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test Scenarios'!$A$1:$G$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$F$189</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test Scenarios'!$A$1:$G$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Proposal vs Built'!$A$1:$E$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -610,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -645,7 +647,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Khavya Sakthivel &amp; Sukumar Dhandapani (Development) · Souvik Das (QA)</t>
+          <t>Khavya Sakthivel &amp; Sukumar Dhandapani (Development) · Souvik Das (QA) — updated 2026-10-22 (sections 18–20 added)</t>
         </is>
       </c>
     </row>
@@ -703,15 +705,15 @@
     </row>
     <row r="13">
       <c r="A13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="C13" s="7">
-        <f>COUNTIF(Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIF(Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="D13" s="7">
@@ -762,15 +764,15 @@
         </is>
       </c>
       <c r="B18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A18,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A18,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A18,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A18,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D18" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A18,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A18,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E18" s="10">
@@ -785,15 +787,15 @@
         </is>
       </c>
       <c r="B19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A19,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A19,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A19,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A19,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A19,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A19,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E19" s="10">
@@ -808,15 +810,15 @@
         </is>
       </c>
       <c r="B20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A20,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A20,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A20,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A20,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D20" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A20,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A20,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E20" s="10">
@@ -831,15 +833,15 @@
         </is>
       </c>
       <c r="B21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A21,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A21,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A21,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A21,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A21,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A21,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E21" s="10">
@@ -854,15 +856,15 @@
         </is>
       </c>
       <c r="B22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A22,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A22,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A22,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A22,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D22" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A22,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A22,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E22" s="10">
@@ -877,15 +879,15 @@
         </is>
       </c>
       <c r="B23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A23,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A23,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A23,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A23,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D23" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A23,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A23,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E23" s="10">
@@ -900,15 +902,15 @@
         </is>
       </c>
       <c r="B24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A24,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A24,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A24,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A24,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D24" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A24,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A24,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E24" s="10">
@@ -923,15 +925,15 @@
         </is>
       </c>
       <c r="B25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A25,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A25,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A25,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A25,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D25" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A25,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A25,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E25" s="10">
@@ -946,15 +948,15 @@
         </is>
       </c>
       <c r="B26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A26,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A26,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A26,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A26,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D26" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A26,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A26,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E26" s="10">
@@ -969,15 +971,15 @@
         </is>
       </c>
       <c r="B27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A27,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A27,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A27,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A27,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D27" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A27,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A27,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E27" s="10">
@@ -992,15 +994,15 @@
         </is>
       </c>
       <c r="B28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A28,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A28,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A28,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A28,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D28" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A28,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A28,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E28" s="10">
@@ -1015,15 +1017,15 @@
         </is>
       </c>
       <c r="B29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A29,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A29,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A29,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A29,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D29" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A29,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A29,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E29" s="10">
@@ -1038,15 +1040,15 @@
         </is>
       </c>
       <c r="B30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A30,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A30,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A30,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A30,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D30" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A30,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A30,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E30" s="10">
@@ -1061,15 +1063,15 @@
         </is>
       </c>
       <c r="B31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A31,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A31,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A31,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A31,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D31" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A31,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A31,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E31" s="10">
@@ -1084,15 +1086,15 @@
         </is>
       </c>
       <c r="B32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A32,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A32,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A32,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A32,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D32" s="10">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A32,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A32,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E32" s="10">
@@ -1107,15 +1109,15 @@
         </is>
       </c>
       <c r="B33">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A33,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A33,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C33">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A33,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A33,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D33">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A33,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A33,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E33">
@@ -1130,19 +1132,88 @@
         </is>
       </c>
       <c r="B34">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A34,Tasks!$D$2:$D$133,"Completed")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A34,Tasks!$D$2:$D$189,"Completed")</f>
         <v/>
       </c>
       <c r="C34">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A34,Tasks!$D$2:$D$133,"In Progress")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A34,Tasks!$D$2:$D$189,"In Progress")</f>
         <v/>
       </c>
       <c r="D34">
-        <f>COUNTIFS(Tasks!$B$2:$B$133,$A34,Tasks!$D$2:$D$133,"Not Started")</f>
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A34,Tasks!$D$2:$D$189,"Not Started")</f>
         <v/>
       </c>
       <c r="E34">
         <f>SUM(B34:D34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="B35">
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A35,Tasks!$D$2:$D$189,"Completed")</f>
+        <v/>
+      </c>
+      <c r="C35">
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A35,Tasks!$D$2:$D$189,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="D35">
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A35,Tasks!$D$2:$D$189,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="E35">
+        <f>SUM(B35:D35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="B36">
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A36,Tasks!$D$2:$D$189,"Completed")</f>
+        <v/>
+      </c>
+      <c r="C36">
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A36,Tasks!$D$2:$D$189,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="D36">
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A36,Tasks!$D$2:$D$189,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="E36">
+        <f>SUM(B36:D36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="B37">
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A37,Tasks!$D$2:$D$189,"Completed")</f>
+        <v/>
+      </c>
+      <c r="C37">
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A37,Tasks!$D$2:$D$189,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="D37">
+        <f>COUNTIFS(Tasks!$B$2:$B$189,$A37,Tasks!$D$2:$D$189,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="E37">
+        <f>SUM(B37:D37)</f>
         <v/>
       </c>
     </row>
@@ -1160,7 +1231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F133"/>
+  <dimension ref="A1:F189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2519,7 +2590,7 @@
       <c r="E53" s="16" t="inlineStr"/>
       <c r="F53" s="17" t="inlineStr">
         <is>
-          <t>Recommended add-on from pain-point research — not yet scoped</t>
+          <t>Recommended add-on from pain-point research — not yet scoped [2026-10-22] A template decline notice (ECOA wording) is shown to borrowers on rejection; a compliant adverse-action notice is tracked in Section 18.</t>
         </is>
       </c>
     </row>
@@ -3577,11 +3648,15 @@
       </c>
       <c r="D95" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E95" s="16" t="inlineStr"/>
-      <c r="F95" s="17" t="inlineStr"/>
+      <c r="F95" s="17" t="inlineStr">
+        <is>
+          <t>Backend suite: 61 tests (verification, statement analysis, RAG grounding, decision rules, borrower-view privacy); 60 pass, 1 pre-existing failure (test/rag/serviceClients.test.js imports a missing export). No frontend or route-level tests yet.</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="30" customHeight="1">
       <c r="A96" s="13" t="n">
@@ -4025,13 +4100,13 @@
       </c>
       <c r="D113" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E113" s="16" t="inlineStr"/>
       <c r="F113" s="17" t="inlineStr">
         <is>
-          <t>New status model, beyond the current submitted/needs-review/approved/rejected enum</t>
+          <t>New status model, beyond the current submitted/needs-review/approved/rejected enum [2026-10-22] A Progress page now shows a derived 6-step timeline (submitted &gt; documents &gt; verification &gt; issues &gt; officer review &gt; decision) with a "You are here" marker. Still missing: a persisted milestone status model and the closing / disbursement stages.</t>
         </is>
       </c>
     </row>
@@ -4536,13 +4611,1413 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>NEEDS FUNDING — real bureau access (Equifax/Experian/TransUnion) requires a licensed FCRA "permissible purpose" relationship, not just an API key; soft-pull aggregators (Array, Bloom Credit, MeridianLink) are the realistic funded path</t>
+          <t>NEEDS FUNDING — real bureau access (Equifax/Experian/TransUnion) requires a licensed FCRA "permissible purpose" relationship, not just an API key; soft-pull aggregators (Array, Bloom Credit, MeridianLink) are the realistic funded path [2026-10-22] Interim: staff enter the credit score by hand on the Decision page (Section 18).</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>7. Frontend — Screens &amp; Navigation</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Verification checklist on the Documents tab — every check (matches and flags) per document, plus an application-wide summary</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>components/VerificationSummary.js. Answers the jury question "what parameters are checked": expected value next to value found, cross-document checks tagged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>7. Frontend — Screens &amp; Navigation</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>One readable URL per application page: /applications/:id/{progress,documents,verification,action-needed,assistant,decision}</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>App.js linking config; browser tab title names the page. AuthContext now waits for the saved session so a reload keeps the deep link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>7. Frontend — Screens &amp; Navigation</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Progress page — % complete, "You are here" timeline, next step</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>ProgressTab.js, utils/progress.js. Derived from documents, verification and status; no new backend state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>7. Frontend — Screens &amp; Navigation</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Action Needed page — open items with one-tap upload / re-upload</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>ActionNeededTab.js; tab shows the open count. Upload logic extracted to utils/uploadDocument.js.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>7. Frontend — Screens &amp; Navigation</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Assistant as a full page, sidebar "Ask LoanLens" entry and per-application sidebar sub-navigation</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>The floating launcher is hidden on the Assistant page (it covered Send). chatBus.js lets the sidebar open the chat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>6. RAG Assistant (Conversational Q&amp;A)</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Chat answers application-state questions from real data and opens the matching page</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>assistantActions.js: documents / progress / verification / action needed (+ decision for staff). No AI credits needed. Questions naming another person go to the server, which enforces access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>6. RAG Assistant (Conversational Q&amp;A)</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Grouped sample questions in the chat (documents, progress, verification, policy; officer and underwriter sets)</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>AssistantTab.js. Policy-source navigation with sentence highlighting is Section 20.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>10. Hosting &amp; Deployment</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Anthropic API credits / billing — IT ticket #2166509</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Key returns HTTP 400 "credit balance too low"; Console shows $0.00 on the Evaluation plan. Blocks live extraction and the AI assistant. backend/check-credits.js reproduces it. Meanwhile use MOCK_AI=true or the Groq provider.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>10. Hosting &amp; Deployment</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Rotate the Anthropic API key (it was visible in a screenshot) and update backend/.env and the Render environment</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Do this once billing is active. The key must only live in .env, never in .env.example.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>12. Documentation</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Reconcile LoanLensAI_RAG_Implementation_Plan.xlsx statuses with the code</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>All 83 tasks read "Not Started" although R2 file storage and several RAG commits landed after 2026-10-02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>12. Documentation</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Ask Rovo / ThoughtFocus mentor questions Q01–Q13 and record the answers</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Rovo Questions sheet of the RAG plan: all 13 still "Open", no answers. Priority: Q01 (approved cloud account), Q02 (third-party policy), Q03/Q04 (tenant isolation), Q06 (approved embeddings), Q09 (RAG evaluation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>12. Documentation</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Document "Proposal vs Built" for the pitch (see the new sheet in this workbook) and the stack deviation (FastAPI/Azure vs Node/Claude)</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Sheet added 2026-10-22; keep it current so the demo never claims an unbuilt feature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Underwriter role — seeded login, not self-registrable, read-only on documents</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>underwriter@loanlens.demo. config/roles.js; self-registration still only offers officer / borrower.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Decision endpoint: approve / decline / refer / return, enforced by role and application state</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>POST /applications/:id/decision; all rules in services/decisionRules.js. Before this, nothing in the app could set approved or rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Policy-parameter assessment: documents, identity, income, credit score, affordability — waivable vs non-waivable</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Only credit score and affordability can be waived. Name / SSN / document-type / income mismatches and missing documents can only be fixed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Credit score entry by staff, locked to whoever currently holds the file</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>PUT /applications/:id/credit-score; manual entry (no bureau pull). Officer before referral, underwriter while referred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Exception approval: waived parameters, compensating factors, "who knows the borrower" note, conditions of approval</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Compensating factors required (20+ chars); every unmet parameter must be named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Append-only audit trail of every review action (who, role, when, note, details)</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Application.reviewHistory; shown on the Decision page. Covers decisions only — extraction events are in Section 19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Borrower-safe view: outcome, reasons or conditions only — never the score, audit trail or exception rationale</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>forViewer() + borrowerNotice(); unit-tested on the real functions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Documents locked while an application is referred or decided</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>documents.js upload / delete return 409; underwriter can preview files but not change them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Staff-only Decision page, "With Underwriter" status, Underwriter portal heading, staff chat questions</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>DecisionTab.js. Tested in the browser against a mock API that uses the real rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Unit tests for decision rules and borrower-view privacy</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>backend/test/decisions/ — 21 tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Confirm the real minimum credit score per product with the bank</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>NEEDS INPUT — 620 (auto) / 660 (personal) / 680 (business) in config/underwriting.js are demo placeholders. Also add the "Credit Checks &amp; Credit Score Policy" document (Section 20).</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Click-through of the full officer &gt; underwriter &gt; borrower flow on real MongoDB</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Only unit tests and a mock API so far. Run npm run reset first (adds the underwriter and Arjun Mehta score 598).</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Add the credit-exception scenario to DEMO_SCRIPT.md</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Arjun Mehta (score 598): officer cannot approve, refers, underwriter approves with an exception, borrower sees only the outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Notify on referral and decision (email / in-app)</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Policy text already promises notification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Underwriter queue view — referred files first, with filters</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Underwriters currently see every application; referred ones show "With Underwriter".</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Approval limits / dual control (second approver above a loan amount)</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Typical bank control; not in the proposal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Appeals — re-open a decided application</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>A decided application is currently immutable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Compliant adverse-action notice (ECOA / Reg B): creditor details, bureau disclosure when a report was used, delivery deadline</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Current notice is generic template wording — needs compliance review. Related to task 52.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>18. Loan Decision &amp; Underwriter Exception Workflow</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Co-signer / guarantor role (borrower-side, liable, submits own documents)</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Different from the underwriter: a person who vouches AND signs. Needs the multi-party model in Section 14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Binder dump: auto-split and classify a large mixed PDF (200–500 pages)</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Headline feature of the submission. Today one upload is treated as one document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>TILA / RESPA disclosure-timing compliance checks</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Promised in the submission; no rule or data exists yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>MISMO-standard JSON output for LOS integration</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Phase 3 in the submission; legitimately later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Cross-document address check (application vs licence / pay stub / bank statement)</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Submission promised name, SSN, income and address. Address is extracted but not compared. Distinct from task 131 (USPS validation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Complete audit trail of every extraction and decision</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Decisions and credit-score entries are logged (Section 18). Uploads, extractions and re-verifications are not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Multi-tenant SaaS: per-bank tenancy and policy indexing</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>RAG plan phase P2; the app is single-bank today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>GLBA / SOC 2-aligned controls: encryption at rest, zero-retention LLM terms, access logging</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Submission risk-mitigation promise; only role-based access exists today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Pay stub / bank statement recency check (policy: within 30 days)</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Policy and FAQ say older documents are rejected; verification.js has no date check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>ID expiry check (policy: expired IDs are not accepted)</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>No expiry field is extracted or checked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Edit an application after submission (FAQ says borrowers can)</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>No edit endpoint or screen exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Reconcile policy text with code: payment ratios (policy 3x / 45% vs code 15% / 20%) and term options</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Answers currently quote the policy numbers, not the ones the system enforces. See docs/POLICY_COVERAGE_AND_QUESTIONS.md section 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Auto loan: capture vehicle value / purchase document for the "110% of book value" rule</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Policy states the limit; no field or document supports it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>19. Proposal Gaps — Promised in Submission, Not Yet Built</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Review policy promises the product does not keep (email notice, rejection of blurry documents)</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Either build the behaviour or reword the policy; list in POLICY_COVERAGE_AND_QUESTIONS.md section 1b.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Check which policy documents are actually live in the admin panel and compare with the required list</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Uploads are stored only as Chroma chunks; GET /rag-admin/documents (admin login) lists them. Not readable from the dev machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Policy document: Interest Rates, Fees &amp; Charges</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Priority 1. Router already sends rate / fee questions to policy; no document exists. Must not quote specific rates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Policy document: Repayment, Prepayment &amp; Foreclosure</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Priority 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Policy document: Credit Checks &amp; Credit Score Policy</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Priority 1. Also supplies the minimum scores used by the underwriter workflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Policy document: Co-signers &amp; Joint Applicants</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Priority 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Policy document: Collateral &amp; Vehicle Requirements (auto)</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Priority 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Policy document: Adverse Action, Denial Reasons &amp; Appeals</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Priority 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Policy documents, priority 2: late payment &amp; hardship, privacy &amp; retention, closing &amp; disbursement, contact &amp; escalation, eligibility by employment type</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>See POLICY_COVERAGE_AND_QUESTIONS.md section 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Remove the "Fictional policy… synthetic content" banner line from every policy file</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>It lands inside the first retrieved chunk and can be quoted in answers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Policy read API: list documents and return chunks in order (any logged-in user)</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Needed by the policy page; getCollectionRecords must also request document text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Policy page: open the cited policy, highlight the matching sentence, link from chat sources and sidebar</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Design in POLICY_COVERAGE_AND_QUESTIONS.md section 5. Open decision: which policies borrowers may see.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>20. Policy Documents &amp; Policy Page</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Add the 55 question scenarios to data/seed/test-questions.md and run them</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Covers policy, own-application, mixed, follow-up, refuse and officer questions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F118"/>
-  <conditionalFormatting sqref="D2:D118">
+  <autoFilter ref="A1:F189"/>
+  <conditionalFormatting sqref="D2:D189">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$D2="Completed"</formula>
     </cfRule>
@@ -4554,7 +6029,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D189" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Completed,In Progress,Not Started"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4568,7 +6043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5597,9 +7072,394 @@
         </is>
       </c>
     </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="13" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Verification checklist</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>Documents tab lists every check, matches and flags</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>Upload any document and look at its card on the Documents tab.</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="inlineStr">
+        <is>
+          <t>A "Verification checks" block shows "N fields extracted · M checks run · X matched · Y flagged" and one row per check with expected vs found. An application-wide summary sits above the documents.</t>
+        </is>
+      </c>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>The jury asked to see which parameters are verified, not only the problems.</t>
+        </is>
+      </c>
+      <c r="G30" s="18" t="inlineStr">
+        <is>
+          <t>Yes — previewed in the browser with sample data; a real upload has not been clicked through</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Page URLs</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>A reload keeps you on the same application page</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>Open /applications/&lt;id&gt;/progress while logged in and reload the browser.</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr">
+        <is>
+          <t>You stay on the Progress page; the tab title reads "LoanLens AI · Application · Progress".</t>
+        </is>
+      </c>
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>Pages can be bookmarked and shared; the chat can open them.</t>
+        </is>
+      </c>
+      <c r="G31" s="18" t="inlineStr">
+        <is>
+          <t>Yes — browser against a mock API</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="13" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Chat navigation</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>"What documents have I uploaded?" opens the Documents page</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>Open the chat and ask the question (or click the sample question).</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="inlineStr">
+        <is>
+          <t>The answer lists the uploaded documents and any still needed, and the Documents page opens with an "Opened Documents" link.</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>Chat becomes a way to navigate, and the answer comes from real data, not the AI.</t>
+        </is>
+      </c>
+      <c r="G32" s="18" t="inlineStr">
+        <is>
+          <t>Yes — browser against a mock API</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="13" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Chat navigation</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>Asking from the Assistant page does not lose the conversation</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>On the Assistant page ask "What is the progress of my application?".</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>The answer stays on the page with an "Open Progress" link instead of navigating away.</t>
+        </is>
+      </c>
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>Navigating would unmount the chat and lose the conversation.</t>
+        </is>
+      </c>
+      <c r="G33" s="18" t="inlineStr">
+        <is>
+          <t>Yes — browser against a mock API</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="13" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Decision workflow</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>Loan officer cannot approve a file whose credit score is below the minimum</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>Record a score of 598 on a personal-loan file (minimum 660) and try to approve.</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>Approve is disabled and the API returns 422 "Refer it to the underwriter for an exception". Referring is offered.</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>The core of the exception process: an officer cannot approve past a parameter.</t>
+        </is>
+      </c>
+      <c r="G34" s="18" t="inlineStr">
+        <is>
+          <t>Yes — unit tests and mock API; not on real MongoDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="13" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>Decision workflow</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>An exception needs a justification, compensating factors and every unmet parameter named</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>As officer refer with a 2-character note; as underwriter approve without compensating factors.</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>Both are refused with a specific message; with proper text the referral and the exception approval succeed.</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>Stops "ok" from being a reason for waiving a bank rule.</t>
+        </is>
+      </c>
+      <c r="G35" s="18" t="inlineStr">
+        <is>
+          <t>Yes — unit tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>Decision workflow</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="inlineStr">
+        <is>
+          <t>A non-waivable mismatch can never be referred or waived</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>Use a file with an SSN or name mismatch and a low credit score; try to refer, then (as underwriter) waive "identity".</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="inlineStr">
+        <is>
+          <t>Referral and waiver are refused: the borrower must correct the mismatch.</t>
+        </is>
+      </c>
+      <c r="F36" s="15" t="inlineStr">
+        <is>
+          <t>An exception is for a short borrower, not for documents that disagree about who the borrower is.</t>
+        </is>
+      </c>
+      <c r="G36" s="18" t="inlineStr">
+        <is>
+          <t>Yes — unit tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="13" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>Decision workflow</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>Credit score cannot be changed after referral by the officer</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>Refer a file, then as officer try to change the score.</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="inlineStr">
+        <is>
+          <t>409; only the underwriter can change it while the file is referred.</t>
+        </is>
+      </c>
+      <c r="F37" s="15" t="inlineStr">
+        <is>
+          <t>The officer must not alter what the underwriter is judging.</t>
+        </is>
+      </c>
+      <c r="G37" s="18" t="inlineStr">
+        <is>
+          <t>Yes — unit tests and mock API</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="13" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Decision workflow</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>Borrower never sees the credit score, audit trail or exception rationale</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>Approve a file as an exception, then fetch it as the borrower.</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="inlineStr">
+        <is>
+          <t>Only the outcome and the conditions are returned; no score, history, waived parameters or relationship note.</t>
+        </is>
+      </c>
+      <c r="F38" s="15" t="inlineStr">
+        <is>
+          <t>Internal rationale and a borrower's credit data must stay with bank staff.</t>
+        </is>
+      </c>
+      <c r="G38" s="18" t="inlineStr">
+        <is>
+          <t>Yes — unit tests on the real functions and mock API</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="13" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>Decision workflow</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>Documents are locked while a file is referred or decided</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>Refer a file, then as the borrower try to upload or delete a document.</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="inlineStr">
+        <is>
+          <t>409 with the reason; the underwriter can still preview files but not change them.</t>
+        </is>
+      </c>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>The documents are the record the decision rests on.</t>
+        </is>
+      </c>
+      <c r="G39" s="18" t="inlineStr">
+        <is>
+          <t>Not yet — implemented in code; needs a live test on real MongoDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="13" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Decision workflow</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>Underwriter login works and cannot be self-registered</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>Run npm run reset, sign in as underwriter@loanlens.demo, then try to register with role underwriter.</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr">
+        <is>
+          <t>Login succeeds with the Underwriter portal heading; registration with that role returns 400.</t>
+        </is>
+      </c>
+      <c r="F40" s="15" t="inlineStr">
+        <is>
+          <t>An approval authority must not be creatable by anyone.</t>
+        </is>
+      </c>
+      <c r="G40" s="18" t="inlineStr">
+        <is>
+          <t>Not yet — needs a live test on real MongoDB</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G29"/>
-  <conditionalFormatting sqref="G2:G29">
+  <autoFilter ref="A1:G40"/>
+  <conditionalFormatting sqref="G2:G40">
     <cfRule type="expression" priority="1" dxfId="3">
       <formula>LEFT($G2,3)="Yes"</formula>
     </cfRule>
@@ -5612,4 +7472,485 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Proposal promise</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>What exists today</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Gap / next step</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Tracker section</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Extract data and cross-verify name, SSN, income, address</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Built, with gaps</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Name, income, employer, SSN last-4, business name, revenue, plus cross-document deposit and payroll-math checks</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>Address is not compared; SSN is last-4 only</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>5, 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Confidence scoring with human-in-the-loop routing</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Low-confidence extractions are flagged for review, never guessed</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Exceptions dashboard</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Action Needed list and page; flags show in the application list</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Officer is the final approver</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Loan officer and underwriter decision workflow with an audit trail</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>Notifications, appeals, real minimum credit scores</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>RAG Q&amp;A with citations for officers and borrowers (web)</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Built, not true RAG</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Policy corpus grounded answers with citations; chat also navigates to pages</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Vector search and per-tenant retrieval; policy page with highlighting</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>6, 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>RAG on WhatsApp</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Webhook, routing into the assistant, outbound replies</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Missing-document detection with one-click borrower email</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Detection built</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>In-app self-service re-upload replaces the email</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>Email notification not built</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>13, 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>"Binder dump": auto-split and classify large mixed PDFs (200–500 pages)</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Not built</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>One upload is one document</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>Page splitting, page-level classification, progress</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>TILA / RESPA disclosure-timing checks</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Not built</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Rules and data model</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>MISMO JSON output for LOS integration</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Not built</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Phase 3 of the submission</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Complete audit trail of every extraction and decision</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Decisions, referrals and credit-score entries are logged; superseded documents kept</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Log uploads and extractions</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>18, 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>GLBA / SOC 2-aligned controls</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>Role-based access; private file storage (R2)</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>Encryption at rest, zero-retention LLM terms, access logging</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Multi-tenant SaaS, per-bank policy indexing</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Not built</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>Single bank</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>RAG plan phase P2</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Residential / consumer loans with 1003 / URLA</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>Different scope</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Auto, personal and small-business loans</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>State the scope change in the pitch</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Azure Document AI / FastAPI / React / vector DB</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Different stack</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Claude vision, Node / Express, Expo, no vector DB yet</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Document the deviation; confirm approved cloud with ThoughtFocus (Rovo Q01)</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Added beyond the proposal</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>Small-business vertical, self-service live exceptions, payroll-math and deposit checks, affordability warning, underwriter exception workflow, mock-AI mode</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>Lead the pitch with the exception and fraud-signal story</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>5, 13, 18</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E17"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: mark Proposal vs Built task complete in the tracker
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LoanLensAI_Development_Task_Tracker.xlsx
+++ b/docs/LoanLensAI_Development_Task_Tracker.xlsx
@@ -636,7 +636,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -658,7 +657,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
@@ -673,7 +671,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -721,8 +718,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
@@ -4906,12 +4901,12 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Sheet added 2026-10-22; keep it current so the demo never claims an unbuilt feature.</t>
+          <t>Sheet added 2026-10-22; keep it current so the demo never claims an unbuilt feature. [2026-10-24] Sheet "Proposal vs Built" is in this workbook; revisit when features land.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Act 2 (identity, credit and the exception) to the demo script
Five borrower stories in demo order, the Arjun exception walk-through
across officer and underwriter, jury Q&A, and recovery tips. Marks the two
demo-script tasks complete in the tracker.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LoanLensAI_Development_Task_Tracker.xlsx
+++ b/docs/LoanLensAI_Development_Task_Tracker.xlsx
@@ -5226,12 +5226,12 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Arjun Mehta (score 598): officer cannot approve, refers, underwriter approves with an exception, borrower sees only the outcome.</t>
+          <t>Arjun Mehta (score 598): officer cannot approve, refers, underwriter approves with an exception, borrower sees only the outcome. [2026-10-24] Added as "Act 2" in docs/DEMO_SCRIPT.md (five stories, exception walk-through, jury Q&amp;A).</t>
         </is>
       </c>
     </row>
@@ -6201,12 +6201,12 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Suggested order is in docs/SIMULATED_VERIFICATION.md.</t>
+          <t>Suggested order is in docs/SIMULATED_VERIFICATION.md. [2026-10-24] Added as "Act 2" in docs/DEMO_SCRIPT.md (five stories, exception walk-through, jury Q&amp;A).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: let borrowers edit a submitted application
PUT /applications/:id for non-identity fields while Submitted/Needs Review;
same intake rules, documents re-verified, every change logged old->new.
Edit button and form on the application page; FAQ and tracker updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LoanLensAI_Development_Task_Tracker.xlsx
+++ b/docs/LoanLensAI_Development_Task_Tracker.xlsx
@@ -5626,12 +5626,12 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>No edit endpoint or screen exists.</t>
+          <t>PUT /applications/:id (borrower, Submitted/Needs Review only). Non-identity fields; same intake rules; all documents re-verified; every change logged old-&gt;new in review history. Edit button + form in ApplicationDetailScreen. 14 unit tests. FAQ updated: re-run /admin/ingest-chroma.</t>
         </is>
       </c>
     </row>

</xml_diff>